<commit_message>
Archivo index-JMJ.js fixes #16
</commit_message>
<xml_diff>
--- a/SOS2526-19-Propuesta.xlsx
+++ b/SOS2526-19-Propuesta.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="176" uniqueCount="131">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="316" uniqueCount="198">
   <si>
     <t>Nombre / enlace repositorio Github</t>
   </si>
@@ -217,6 +217,12 @@
     <t>Afghanistan</t>
   </si>
   <si>
+    <t>########</t>
+  </si>
+  <si>
+    <t>6,4</t>
+  </si>
+  <si>
     <t>magnitude 6.4M and depth 0km</t>
   </si>
   <si>
@@ -238,34 +244,235 @@
     <t>460000 people within 100km</t>
   </si>
   <si>
-    <t>"[58.175, 35.217]",Earthquake in Iran,Earthquake in Iran,Green M 4.9 Earthquake in Iran at: 14 Feb 2000 00:00:00.,Green,1,Green,0.5,Iran,2000-02-14T00:00:00,2000-02-14T00:00:00,4.9,magnitude 4.9M and depth 0km,NEIC,IRN,EQ,4.9M,0 Km,440000 people within 100km,</t>
+    <t>[58.175, 35.217]</t>
   </si>
   <si>
-    <t>"[58.218, 35.288]",Earthquake in Iran,Earthquake in Iran,Green M 5.3 Earthquake in Iran at: 03 Feb 2000 00:00:00.,Green,1,Green,0.5,Iran,2000-02-03T00:00:00,2000-02-03T00:00:00,5.3,magnitude 5.3M and depth 0km,NEIC,IRN,EQ,5.3M,0 Km,470000 people within 100km,</t>
+    <t>Earthquake in Iran</t>
   </si>
   <si>
-    <t>"[25.69, 34.22]","Earthquake in Crete, Greece","Earthquake in Crete, Greece","Green M 5.5 Earthquake in Crete, Greece at: 05 Apr 2000 04:37:00.",Green,1,Green,0.0,"Crete, Greece",2000-04-05T04:37:00,2000-04-05T04:37:00,5.5,"Magnitude 5.5M, Depth:10km",NGDC,,EQ,5.5M,10 Km,30 thousand in MMI IV,1.1 ()</t>
+    <t>Green M 4.9 Earthquake in Iran at: 14 Feb 2000 00:00:00.</t>
   </si>
   <si>
-    <t>"[123.573, -1.105]",Earthquake in Indonesia,Earthquake in Indonesia,Orange M 7.6 Earthquake in Indonesia at: 04 May 2000 04:21:00.,Orange,2,Orange,1.5,Indonesia,2000-05-04T04:21:00,2000-05-04T04:21:00,7.6,"Magnitude 7.6M, Depth:10km",NGDC,IDN,EQ,7.6M,10 Km,90 thousand (in MMI&gt;=VII),4.8 (Indonesia)</t>
+    <t>Green</t>
   </si>
   <si>
-    <t>"[97.453, -13.802]",Earthquake in South Indian Ocean,Earthquake in South Indian Ocean,Orange M 7.9 Earthquake in South Indian Ocean at: 18 Jun 2000 14:44:00.,Orange,2,Orange,1.05,South Indian Ocean,2000-06-18T14:44:00,2000-06-18T14:44:00,7.9,"Magnitude 7.9M, Depth:10km",NGDC,,EQ,7.9M,10 Km,Few people affected (in MMI&gt;=VII),1.1 ()</t>
+    <t>Iran</t>
   </si>
   <si>
-    <t>"[139.376, 33.901]","Earthquake in Southeast Of Honshu, Japan","Earthquake in Southeast Of Honshu, Japan","Green M 6.5 Earthquake in Southeast Of Honshu, Japan at: 30 Jul 2000 12:25:00.",Green,1,Green,0.5,"Southeast Of Honshu, Japan",2000-07-30T12:25:00,2000-07-30T12:25:00,6.5,"Magnitude 6.5M, Depth:10km",NGDC,,EQ,6.5M,10 Km,3 thousand in MMI VI,1.1 ()</t>
+    <t>magnitude 4.9M and depth 0km</t>
   </si>
   <si>
-    <t>"[139.26, 34.319]","Earthquake in Near S. Coast Of Honshu, Japan","Earthquake in Near S. Coast Of Honshu, Japan","Green M 6.1 Earthquake in Near S. Coast Of Honshu, Japan at: 15 Jul 2000 01:30:00.",Green,1,Green,0.5,"Near S. Coast Of Honshu, Japan",2000-07-15T01:30:00,2000-07-15T01:30:00,6.1,"Magnitude 6.1M, Depth:10km",NGDC,,EQ,6.1M,10 Km,3 thousand (in MMI&gt;=VII),1.1 ()</t>
+    <t>IRN</t>
   </si>
   <si>
-    <t>"[139.131, 34.221]","Earthquake in Near S. Coast Of Honshu, Japan","Earthquake in Near S. Coast Of Honshu, Japan","Green M 6.1 Earthquake in Near S. Coast Of Honshu, Japan at: 01 Jul 2000 07:01:00.",Green,1,Green,0.5,"Near S. Coast Of Honshu, Japan",2000-07-01T07:01:00,2000-07-01T07:01:00,6.1,"Magnitude 6.1M, Depth:10km",NGDC,,EQ,6.1M,10 Km,2 thousand (in MMI&gt;=VII),1.1 ()</t>
+    <t>4.9M</t>
   </si>
   <si>
-    <t>"[69.425, 37.451]",Earthquake in Tajikistan,Earthquake in Tajikistan,Green M 4.8 Earthquake in Tajikistan at: 31 Oct 2000 00:00:00.,Green,1,Green,0.5,Tajikistan,2000-10-31T00:00:00,2000-10-31T00:00:00,4.8,magnitude 4.8M and depth 0km,NEIC,TJK,EQ,4.8M,0 Km,3430000 people within 100km,</t>
+    <t>440000 people within 100km</t>
   </si>
   <si>
-    <t>"[152.327, -4.001]",Earthquake in Papua New Guinea,Earthquake in Papua New Guinea,Red M 8 Earthquake in Papua New Guinea at: 16 Nov 2000 04:54:00.,Red,3,Red,3.425,Papua New Guinea,2000-11-16T04:54:00,2000-11-16T04:54:00,8.0,"Magnitude 8M, Depth:10km",NGDC,PNG,EQ,8.0M,10 Km,140 thousand (in MMI&gt;=VII),7.6 (Papua New Guinea)</t>
+    <t>[58.218, 35.288]</t>
+  </si>
+  <si>
+    <t>Green M 5.3 Earthquake in Iran at: 03 Feb 2000 00:00:00.</t>
+  </si>
+  <si>
+    <t>magnitude 5.3M and depth 0km</t>
+  </si>
+  <si>
+    <t>5.3M</t>
+  </si>
+  <si>
+    <t>470000 people within 100km</t>
+  </si>
+  <si>
+    <t>[25.69, 34.22]</t>
+  </si>
+  <si>
+    <t>Earthquake in Crete, Greece</t>
+  </si>
+  <si>
+    <t>Green M 5.5 Earthquake in Crete, Greece at: 05 Apr 2000 04:37:00.</t>
+  </si>
+  <si>
+    <t>Crete, Greece</t>
+  </si>
+  <si>
+    <t>Magnitude 5.5M, Depth:10km</t>
+  </si>
+  <si>
+    <t>NGDC</t>
+  </si>
+  <si>
+    <t>GRC</t>
+  </si>
+  <si>
+    <t>5.5M</t>
+  </si>
+  <si>
+    <t>10 Km</t>
+  </si>
+  <si>
+    <t>30 thousand in MMI IV</t>
+  </si>
+  <si>
+    <t>1.1 ()</t>
+  </si>
+  <si>
+    <t>[123.573, -1.105]</t>
+  </si>
+  <si>
+    <t>Earthquake in Indonesia</t>
+  </si>
+  <si>
+    <t>Orange M 7.6 Earthquake in Indonesia at: 04 May 2000 04:21:00.</t>
+  </si>
+  <si>
+    <t>Orange</t>
+  </si>
+  <si>
+    <t>Indonesia</t>
+  </si>
+  <si>
+    <t>Magnitude 7.6M, Depth:10km</t>
+  </si>
+  <si>
+    <t>IDN</t>
+  </si>
+  <si>
+    <t>7.6M</t>
+  </si>
+  <si>
+    <t>90 thousand (in MMI&gt;=VII)</t>
+  </si>
+  <si>
+    <t>4.8 (Indonesia)</t>
+  </si>
+  <si>
+    <t>[97.453, -13.802]</t>
+  </si>
+  <si>
+    <t>Earthquake in South Indian Ocean</t>
+  </si>
+  <si>
+    <t>Orange M 7.9 Earthquake in South Indian Ocean at: 18 Jun 2000 14:44:00.</t>
+  </si>
+  <si>
+    <t>South Indian Ocean</t>
+  </si>
+  <si>
+    <t>Magnitude 7.9M, Depth:10km</t>
+  </si>
+  <si>
+    <t>7.9M</t>
+  </si>
+  <si>
+    <t>Few people affected (in MMI&gt;=VII)</t>
+  </si>
+  <si>
+    <t>[139.376, 33.901]</t>
+  </si>
+  <si>
+    <t>Earthquake in Southeast Of Honshu, Japan</t>
+  </si>
+  <si>
+    <t>Green M 6.5 Earthquake in Southeast Of Honshu, Japan at: 30 Jul 2000 12:25:00.</t>
+  </si>
+  <si>
+    <t>Southeast Of Honshu, Japan</t>
+  </si>
+  <si>
+    <t>Magnitude 6.5M, Depth:10km</t>
+  </si>
+  <si>
+    <t>JPN</t>
+  </si>
+  <si>
+    <t>6.5M</t>
+  </si>
+  <si>
+    <t>3 thousand in MMI VI</t>
+  </si>
+  <si>
+    <t>[139.26, 34.319]</t>
+  </si>
+  <si>
+    <t>Earthquake in Near S. Coast Of Honshu, Japan</t>
+  </si>
+  <si>
+    <t>Green M 6.1 Earthquake in Near S. Coast Of Honshu, Japan at: 15 Jul 2000 01:30:00.</t>
+  </si>
+  <si>
+    <t>Near S. Coast Of Honshu, Japan</t>
+  </si>
+  <si>
+    <t>Magnitude 6.1M, Depth:10km</t>
+  </si>
+  <si>
+    <t>6.1M</t>
+  </si>
+  <si>
+    <t>3 thousand (in MMI&gt;=VII)</t>
+  </si>
+  <si>
+    <t>[139.131, 34.221]</t>
+  </si>
+  <si>
+    <t>Green M 6.1 Earthquake in Near S. Coast Of Honshu, Japan at: 01 Jul 2000 07:01:00.</t>
+  </si>
+  <si>
+    <t>2 thousand (in MMI&gt;=VII)</t>
+  </si>
+  <si>
+    <t>[69.425, 37.451]</t>
+  </si>
+  <si>
+    <t>Earthquake in Tajikistan</t>
+  </si>
+  <si>
+    <t>Green M 4.8 Earthquake in Tajikistan at: 31 Oct 2000 00:00:00.</t>
+  </si>
+  <si>
+    <t>Tajikistan</t>
+  </si>
+  <si>
+    <t>magnitude 4.8M and depth 0km</t>
+  </si>
+  <si>
+    <t>TJK</t>
+  </si>
+  <si>
+    <t>4.8M</t>
+  </si>
+  <si>
+    <t>3430000 people within 100km</t>
+  </si>
+  <si>
+    <t>[152.327, -4.001]</t>
+  </si>
+  <si>
+    <t>Earthquake in Papua New Guinea</t>
+  </si>
+  <si>
+    <t>Red M 8 Earthquake in Papua New Guinea at: 16 Nov 2000 04:54:00.</t>
+  </si>
+  <si>
+    <t>Papua New Guinea</t>
+  </si>
+  <si>
+    <t>Magnitude 8M, Depth:10km</t>
+  </si>
+  <si>
+    <t>PNG</t>
+  </si>
+  <si>
+    <t>8.0M</t>
+  </si>
+  <si>
+    <t>140 thousand (in MMI&gt;=VII)</t>
+  </si>
+  <si>
+    <t>7.6 (Papua New Guinea)</t>
   </si>
   <si>
     <t>alert_level</t>
@@ -305,9 +512,6 @@
   </si>
   <si>
     <t>Green Drought in Germany, Denmark, France, Latvia, Poland, Sweden from: 21 Jul 2017  to: 09 Feb 2019 .</t>
-  </si>
-  <si>
-    <t>Green</t>
   </si>
   <si>
     <t>Germany</t>
@@ -370,9 +574,6 @@
     <t>Orange Drought in Australia from: 21 Feb 2018  to: 24 Nov 2018 .</t>
   </si>
   <si>
-    <t>Orange</t>
-  </si>
-  <si>
     <t>Australia</t>
   </si>
   <si>
@@ -418,7 +619,7 @@
     <numFmt numFmtId="165" formatCode="0.###############"/>
     <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="10">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -457,6 +658,11 @@
       <name val="Calibri"/>
     </font>
     <font/>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -492,7 +698,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="32">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -552,11 +758,20 @@
       <alignment horizontal="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="top" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment readingOrder="0"/>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="166" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
@@ -569,6 +784,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" wrapText="1"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment shrinkToFit="0" wrapText="1"/>
@@ -28808,115 +29026,682 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="22" t="s">
         <v>62</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="22" t="s">
         <v>63</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="F2" s="21">
+      <c r="F2" s="23">
         <v>3.0</v>
       </c>
-      <c r="G2" s="21" t="s">
+      <c r="G2" s="22" t="s">
         <v>65</v>
       </c>
-      <c r="H2" s="21">
+      <c r="H2" s="23">
         <v>3.0</v>
       </c>
-      <c r="I2" s="21" t="s">
+      <c r="I2" s="22" t="s">
         <v>66</v>
       </c>
-      <c r="J2" s="22">
-        <v>36544.0</v>
-      </c>
-      <c r="K2" s="22">
-        <v>36544.0</v>
-      </c>
-      <c r="L2" s="21">
-        <v>6.4</v>
-      </c>
-      <c r="M2" s="21" t="s">
+      <c r="J2" s="24" t="s">
         <v>67</v>
       </c>
-      <c r="N2" s="21" t="s">
+      <c r="K2" s="24" t="s">
+        <v>67</v>
+      </c>
+      <c r="L2" s="23" t="s">
         <v>68</v>
       </c>
-      <c r="O2" s="21" t="s">
+      <c r="M2" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="P2" s="21" t="s">
+      <c r="N2" s="22" t="s">
         <v>70</v>
       </c>
-      <c r="Q2" s="21" t="s">
+      <c r="O2" s="22" t="s">
         <v>71</v>
       </c>
-      <c r="R2" s="21" t="s">
+      <c r="P2" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="S2" s="21" t="s">
+      <c r="Q2" s="22" t="s">
         <v>73</v>
       </c>
+      <c r="R2" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="S2" s="22" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="21" t="s">
+      <c r="A3" s="22" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="C3" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="D3" s="22" t="s">
+        <v>78</v>
+      </c>
+      <c r="E3" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="F3" s="22">
+        <v>1.0</v>
+      </c>
+      <c r="G3" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="H3" s="22">
+        <v>0.5</v>
+      </c>
+      <c r="I3" s="22" t="s">
+        <v>80</v>
+      </c>
+      <c r="J3" s="25">
+        <v>36570.0</v>
+      </c>
+      <c r="K3" s="25">
+        <v>36570.0</v>
+      </c>
+      <c r="L3" s="22">
+        <v>4.9</v>
+      </c>
+      <c r="M3" s="22" t="s">
+        <v>81</v>
+      </c>
+      <c r="N3" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="O3" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="P3" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q3" s="22" t="s">
+        <v>83</v>
+      </c>
+      <c r="R3" s="22" t="s">
         <v>74</v>
       </c>
+      <c r="S3" s="22" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="21" t="s">
-        <v>75</v>
+      <c r="A4" s="22" t="s">
+        <v>85</v>
+      </c>
+      <c r="B4" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="C4" s="22" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="F4" s="22">
+        <v>1.0</v>
+      </c>
+      <c r="G4" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="H4" s="22">
+        <v>0.5</v>
+      </c>
+      <c r="I4" s="22" t="s">
+        <v>80</v>
+      </c>
+      <c r="J4" s="25">
+        <v>36559.0</v>
+      </c>
+      <c r="K4" s="25">
+        <v>36559.0</v>
+      </c>
+      <c r="L4" s="22">
+        <v>5.3</v>
+      </c>
+      <c r="M4" s="22" t="s">
+        <v>87</v>
+      </c>
+      <c r="N4" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="O4" s="22" t="s">
+        <v>82</v>
+      </c>
+      <c r="P4" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q4" s="22" t="s">
+        <v>88</v>
+      </c>
+      <c r="R4" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="S4" s="22" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="s">
-        <v>76</v>
+      <c r="A5" s="22" t="s">
+        <v>90</v>
+      </c>
+      <c r="B5" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="C5" s="22" t="s">
+        <v>91</v>
+      </c>
+      <c r="D5" s="22" t="s">
+        <v>92</v>
+      </c>
+      <c r="E5" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="F5" s="22">
+        <v>1.0</v>
+      </c>
+      <c r="G5" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="H5" s="22">
+        <v>0.0</v>
+      </c>
+      <c r="I5" s="22" t="s">
+        <v>93</v>
+      </c>
+      <c r="J5" s="25">
+        <v>36621.19236111111</v>
+      </c>
+      <c r="K5" s="25">
+        <v>36621.19236111111</v>
+      </c>
+      <c r="L5" s="22">
+        <v>5.5</v>
+      </c>
+      <c r="M5" s="22" t="s">
+        <v>94</v>
+      </c>
+      <c r="N5" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="O5" s="22" t="s">
+        <v>96</v>
+      </c>
+      <c r="P5" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q5" s="22" t="s">
+        <v>97</v>
+      </c>
+      <c r="R5" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="S5" s="22" t="s">
+        <v>99</v>
+      </c>
+      <c r="T5" s="22" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="s">
-        <v>77</v>
+      <c r="A6" s="22" t="s">
+        <v>101</v>
+      </c>
+      <c r="B6" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="C6" s="22" t="s">
+        <v>102</v>
+      </c>
+      <c r="D6" s="22" t="s">
+        <v>103</v>
+      </c>
+      <c r="E6" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="F6" s="22">
+        <v>2.0</v>
+      </c>
+      <c r="G6" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="H6" s="22">
+        <v>1.5</v>
+      </c>
+      <c r="I6" s="22" t="s">
+        <v>105</v>
+      </c>
+      <c r="J6" s="25">
+        <v>36650.18125</v>
+      </c>
+      <c r="K6" s="25">
+        <v>36650.18125</v>
+      </c>
+      <c r="L6" s="22">
+        <v>7.6</v>
+      </c>
+      <c r="M6" s="22" t="s">
+        <v>106</v>
+      </c>
+      <c r="N6" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="O6" s="22" t="s">
+        <v>107</v>
+      </c>
+      <c r="P6" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q6" s="22" t="s">
+        <v>108</v>
+      </c>
+      <c r="R6" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="S6" s="22" t="s">
+        <v>109</v>
+      </c>
+      <c r="T6" s="22" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="s">
-        <v>78</v>
+      <c r="A7" s="22" t="s">
+        <v>111</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="C7" s="22" t="s">
+        <v>112</v>
+      </c>
+      <c r="D7" s="22" t="s">
+        <v>113</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="F7" s="22">
+        <v>2.0</v>
+      </c>
+      <c r="G7" s="22" t="s">
+        <v>104</v>
+      </c>
+      <c r="H7" s="22">
+        <v>1.05</v>
+      </c>
+      <c r="I7" s="22" t="s">
+        <v>114</v>
+      </c>
+      <c r="J7" s="25">
+        <v>36695.61388888889</v>
+      </c>
+      <c r="K7" s="25">
+        <v>36695.61388888889</v>
+      </c>
+      <c r="L7" s="22">
+        <v>7.9</v>
+      </c>
+      <c r="M7" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="N7" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="O7" s="22" t="s">
+        <v>107</v>
+      </c>
+      <c r="P7" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q7" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="R7" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="S7" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="T7" s="22" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="21" t="s">
+      <c r="A8" s="22" t="s">
+        <v>118</v>
+      </c>
+      <c r="B8" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="C8" s="22" t="s">
+        <v>119</v>
+      </c>
+      <c r="D8" s="22" t="s">
+        <v>120</v>
+      </c>
+      <c r="E8" s="22" t="s">
         <v>79</v>
       </c>
+      <c r="F8" s="22">
+        <v>1.0</v>
+      </c>
+      <c r="G8" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="H8" s="22">
+        <v>0.5</v>
+      </c>
+      <c r="I8" s="22" t="s">
+        <v>121</v>
+      </c>
+      <c r="J8" s="25">
+        <v>36737.51736111111</v>
+      </c>
+      <c r="K8" s="25">
+        <v>36737.51736111111</v>
+      </c>
+      <c r="L8" s="22">
+        <v>6.5</v>
+      </c>
+      <c r="M8" s="22" t="s">
+        <v>122</v>
+      </c>
+      <c r="N8" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="O8" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="P8" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q8" s="22" t="s">
+        <v>124</v>
+      </c>
+      <c r="R8" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="S8" s="22" t="s">
+        <v>125</v>
+      </c>
+      <c r="T8" s="22" t="s">
+        <v>100</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="21" t="s">
-        <v>80</v>
+      <c r="A9" s="22" t="s">
+        <v>126</v>
+      </c>
+      <c r="B9" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="C9" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="D9" s="22" t="s">
+        <v>128</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="F9" s="22">
+        <v>1.0</v>
+      </c>
+      <c r="G9" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="H9" s="22">
+        <v>0.5</v>
+      </c>
+      <c r="I9" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="J9" s="25">
+        <v>36722.0625</v>
+      </c>
+      <c r="K9" s="25">
+        <v>36722.0625</v>
+      </c>
+      <c r="L9" s="22">
+        <v>6.1</v>
+      </c>
+      <c r="M9" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="N9" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="O9" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="P9" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q9" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="R9" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="S9" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="T9" s="22" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="s">
-        <v>81</v>
+      <c r="A10" s="22" t="s">
+        <v>133</v>
+      </c>
+      <c r="B10" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="C10" s="22" t="s">
+        <v>127</v>
+      </c>
+      <c r="D10" s="22" t="s">
+        <v>134</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="F10" s="22">
+        <v>1.0</v>
+      </c>
+      <c r="G10" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="H10" s="22">
+        <v>0.5</v>
+      </c>
+      <c r="I10" s="22" t="s">
+        <v>129</v>
+      </c>
+      <c r="J10" s="25">
+        <v>36708.29236111111</v>
+      </c>
+      <c r="K10" s="25">
+        <v>36708.29236111111</v>
+      </c>
+      <c r="L10" s="22">
+        <v>6.1</v>
+      </c>
+      <c r="M10" s="22" t="s">
+        <v>130</v>
+      </c>
+      <c r="N10" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="O10" s="22" t="s">
+        <v>123</v>
+      </c>
+      <c r="P10" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q10" s="22" t="s">
+        <v>131</v>
+      </c>
+      <c r="R10" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="S10" s="22" t="s">
+        <v>135</v>
+      </c>
+      <c r="T10" s="22" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="s">
-        <v>82</v>
+      <c r="A11" s="22" t="s">
+        <v>136</v>
+      </c>
+      <c r="B11" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="C11" s="22" t="s">
+        <v>137</v>
+      </c>
+      <c r="D11" s="22" t="s">
+        <v>138</v>
+      </c>
+      <c r="E11" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="F11" s="22">
+        <v>1.0</v>
+      </c>
+      <c r="G11" s="22" t="s">
+        <v>79</v>
+      </c>
+      <c r="H11" s="22">
+        <v>0.5</v>
+      </c>
+      <c r="I11" s="22" t="s">
+        <v>139</v>
+      </c>
+      <c r="J11" s="25">
+        <v>36830.0</v>
+      </c>
+      <c r="K11" s="25">
+        <v>36830.0</v>
+      </c>
+      <c r="L11" s="22">
+        <v>4.8</v>
+      </c>
+      <c r="M11" s="22" t="s">
+        <v>140</v>
+      </c>
+      <c r="N11" s="22" t="s">
+        <v>70</v>
+      </c>
+      <c r="O11" s="22" t="s">
+        <v>141</v>
+      </c>
+      <c r="P11" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q11" s="22" t="s">
+        <v>142</v>
+      </c>
+      <c r="R11" s="22" t="s">
+        <v>74</v>
+      </c>
+      <c r="S11" s="22" t="s">
+        <v>143</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="s">
-        <v>83</v>
+      <c r="A12" s="22" t="s">
+        <v>144</v>
+      </c>
+      <c r="B12" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>145</v>
+      </c>
+      <c r="D12" s="22" t="s">
+        <v>146</v>
+      </c>
+      <c r="E12" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="F12" s="22">
+        <v>3.0</v>
+      </c>
+      <c r="G12" s="22" t="s">
+        <v>65</v>
+      </c>
+      <c r="H12" s="22">
+        <v>3.425</v>
+      </c>
+      <c r="I12" s="22" t="s">
+        <v>147</v>
+      </c>
+      <c r="J12" s="25">
+        <v>36846.20416666667</v>
+      </c>
+      <c r="K12" s="25">
+        <v>36846.20416666667</v>
+      </c>
+      <c r="L12" s="22">
+        <v>8.0</v>
+      </c>
+      <c r="M12" s="22" t="s">
+        <v>148</v>
+      </c>
+      <c r="N12" s="22" t="s">
+        <v>95</v>
+      </c>
+      <c r="O12" s="22" t="s">
+        <v>149</v>
+      </c>
+      <c r="P12" s="22" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q12" s="22" t="s">
+        <v>150</v>
+      </c>
+      <c r="R12" s="22" t="s">
+        <v>98</v>
+      </c>
+      <c r="S12" s="22" t="s">
+        <v>151</v>
+      </c>
+      <c r="T12" s="22" t="s">
+        <v>152</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="S2:T2"/>
+    <mergeCell ref="S3:T3"/>
+    <mergeCell ref="S4:T4"/>
+    <mergeCell ref="S11:T11"/>
+  </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -28944,1484 +29729,1484 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="B1" s="23" t="s">
-        <v>84</v>
-      </c>
-      <c r="C1" s="23" t="s">
-        <v>85</v>
-      </c>
-      <c r="D1" s="23" t="s">
-        <v>86</v>
-      </c>
-      <c r="E1" s="23" t="s">
+      <c r="B1" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="C1" s="26" t="s">
+        <v>154</v>
+      </c>
+      <c r="D1" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="E1" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="F1" s="23" t="s">
-        <v>87</v>
-      </c>
-      <c r="G1" s="23" t="s">
-        <v>88</v>
-      </c>
-      <c r="H1" s="23" t="s">
-        <v>89</v>
-      </c>
-      <c r="I1" s="23" t="s">
-        <v>90</v>
-      </c>
-      <c r="J1" s="23" t="s">
-        <v>91</v>
-      </c>
-      <c r="K1" s="23" t="s">
-        <v>92</v>
-      </c>
-      <c r="L1" s="23" t="s">
-        <v>93</v>
-      </c>
-      <c r="M1" s="23" t="s">
-        <v>94</v>
-      </c>
-      <c r="N1" s="23" t="s">
-        <v>95</v>
+      <c r="F1" s="26" t="s">
+        <v>156</v>
+      </c>
+      <c r="G1" s="26" t="s">
+        <v>157</v>
+      </c>
+      <c r="H1" s="26" t="s">
+        <v>158</v>
+      </c>
+      <c r="I1" s="26" t="s">
+        <v>159</v>
+      </c>
+      <c r="J1" s="26" t="s">
+        <v>160</v>
+      </c>
+      <c r="K1" s="26" t="s">
+        <v>161</v>
+      </c>
+      <c r="L1" s="26" t="s">
+        <v>162</v>
+      </c>
+      <c r="M1" s="26" t="s">
+        <v>163</v>
+      </c>
+      <c r="N1" s="26" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="24" t="s">
-        <v>96</v>
-      </c>
-      <c r="B2" s="25" t="s">
-        <v>97</v>
-      </c>
-      <c r="C2" s="25">
+      <c r="A2" s="27" t="s">
+        <v>165</v>
+      </c>
+      <c r="B2" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="C2" s="28">
         <v>1.0</v>
       </c>
-      <c r="D2" s="25">
+      <c r="D2" s="28">
         <v>0.25</v>
       </c>
-      <c r="E2" s="24" t="s">
-        <v>98</v>
-      </c>
-      <c r="F2" s="25">
+      <c r="E2" s="27" t="s">
+        <v>166</v>
+      </c>
+      <c r="F2" s="28">
         <v>2017.0</v>
       </c>
-      <c r="G2" s="25">
+      <c r="G2" s="28">
         <v>2019.0</v>
       </c>
-      <c r="H2" s="25">
+      <c r="H2" s="28">
         <v>80936.0</v>
       </c>
-      <c r="I2" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="J2" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="K2" s="25">
+      <c r="I2" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="J2" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="K2" s="28">
         <v>569.0</v>
       </c>
-      <c r="L2" s="25" t="s">
-        <v>101</v>
-      </c>
-      <c r="M2" s="25">
+      <c r="L2" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="M2" s="28">
         <v>11.087</v>
       </c>
-      <c r="N2" s="25">
+      <c r="N2" s="28">
         <v>53.882</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="24" t="s">
-        <v>96</v>
-      </c>
-      <c r="B3" s="25" t="s">
-        <v>97</v>
-      </c>
-      <c r="C3" s="25">
+      <c r="A3" s="27" t="s">
+        <v>165</v>
+      </c>
+      <c r="B3" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="C3" s="28">
         <v>1.0</v>
       </c>
-      <c r="D3" s="25">
+      <c r="D3" s="28">
         <v>0.25</v>
       </c>
-      <c r="E3" s="24" t="s">
-        <v>102</v>
-      </c>
-      <c r="F3" s="25">
+      <c r="E3" s="27" t="s">
+        <v>170</v>
+      </c>
+      <c r="F3" s="28">
         <v>2017.0</v>
       </c>
-      <c r="G3" s="25">
+      <c r="G3" s="28">
         <v>2019.0</v>
       </c>
-      <c r="H3" s="25">
+      <c r="H3" s="28">
         <v>80936.0</v>
       </c>
-      <c r="I3" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="J3" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="K3" s="25">
+      <c r="I3" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="J3" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="K3" s="28">
         <v>569.0</v>
       </c>
-      <c r="L3" s="25" t="s">
-        <v>101</v>
-      </c>
-      <c r="M3" s="25">
+      <c r="L3" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="M3" s="28">
         <v>11.087</v>
       </c>
-      <c r="N3" s="25">
+      <c r="N3" s="28">
         <v>53.882</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="s">
-        <v>96</v>
-      </c>
-      <c r="B4" s="25" t="s">
-        <v>97</v>
-      </c>
-      <c r="C4" s="25">
+      <c r="A4" s="27" t="s">
+        <v>165</v>
+      </c>
+      <c r="B4" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="C4" s="28">
         <v>1.0</v>
       </c>
-      <c r="D4" s="25">
+      <c r="D4" s="28">
         <v>0.25</v>
       </c>
-      <c r="E4" s="24" t="s">
-        <v>103</v>
-      </c>
-      <c r="F4" s="25">
+      <c r="E4" s="27" t="s">
+        <v>171</v>
+      </c>
+      <c r="F4" s="28">
         <v>2017.0</v>
       </c>
-      <c r="G4" s="25">
+      <c r="G4" s="28">
         <v>2019.0</v>
       </c>
-      <c r="H4" s="25">
+      <c r="H4" s="28">
         <v>80936.0</v>
       </c>
-      <c r="I4" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="J4" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="K4" s="25">
+      <c r="I4" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="J4" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="K4" s="28">
         <v>569.0</v>
       </c>
-      <c r="L4" s="25" t="s">
-        <v>101</v>
-      </c>
-      <c r="M4" s="25">
+      <c r="L4" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="M4" s="28">
         <v>11.087</v>
       </c>
-      <c r="N4" s="25">
+      <c r="N4" s="28">
         <v>53.882</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="24" t="s">
-        <v>96</v>
-      </c>
-      <c r="B5" s="25" t="s">
-        <v>97</v>
-      </c>
-      <c r="C5" s="25">
+      <c r="A5" s="27" t="s">
+        <v>165</v>
+      </c>
+      <c r="B5" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="28">
         <v>1.0</v>
       </c>
-      <c r="D5" s="25">
+      <c r="D5" s="28">
         <v>0.25</v>
       </c>
-      <c r="E5" s="24" t="s">
+      <c r="E5" s="27" t="s">
+        <v>172</v>
+      </c>
+      <c r="F5" s="28">
+        <v>2017.0</v>
+      </c>
+      <c r="G5" s="28">
+        <v>2019.0</v>
+      </c>
+      <c r="H5" s="28">
+        <v>80936.0</v>
+      </c>
+      <c r="I5" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="J5" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="K5" s="28">
+        <v>569.0</v>
+      </c>
+      <c r="L5" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="M5" s="28">
+        <v>11.087</v>
+      </c>
+      <c r="N5" s="28">
+        <v>53.882</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="27" t="s">
+        <v>165</v>
+      </c>
+      <c r="B6" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="C6" s="28">
+        <v>1.0</v>
+      </c>
+      <c r="D6" s="28">
+        <v>0.25</v>
+      </c>
+      <c r="E6" s="27" t="s">
+        <v>173</v>
+      </c>
+      <c r="F6" s="28">
+        <v>2017.0</v>
+      </c>
+      <c r="G6" s="28">
+        <v>2019.0</v>
+      </c>
+      <c r="H6" s="28">
+        <v>80936.0</v>
+      </c>
+      <c r="I6" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="J6" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="K6" s="28">
+        <v>569.0</v>
+      </c>
+      <c r="L6" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="M6" s="28">
+        <v>11.087</v>
+      </c>
+      <c r="N6" s="28">
+        <v>53.882</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="27" t="s">
+        <v>165</v>
+      </c>
+      <c r="B7" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="C7" s="28">
+        <v>1.0</v>
+      </c>
+      <c r="D7" s="28">
+        <v>0.25</v>
+      </c>
+      <c r="E7" s="27" t="s">
+        <v>174</v>
+      </c>
+      <c r="F7" s="28">
+        <v>2017.0</v>
+      </c>
+      <c r="G7" s="28">
+        <v>2019.0</v>
+      </c>
+      <c r="H7" s="28">
+        <v>80936.0</v>
+      </c>
+      <c r="I7" s="28" t="s">
+        <v>167</v>
+      </c>
+      <c r="J7" s="28" t="s">
+        <v>168</v>
+      </c>
+      <c r="K7" s="28">
+        <v>569.0</v>
+      </c>
+      <c r="L7" s="28" t="s">
+        <v>169</v>
+      </c>
+      <c r="M7" s="28">
+        <v>11.087</v>
+      </c>
+      <c r="N7" s="28">
+        <v>53.882</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="29" t="s">
+        <v>175</v>
+      </c>
+      <c r="B8" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="C8" s="28">
+        <v>1.0</v>
+      </c>
+      <c r="D8" s="28">
+        <v>0.75</v>
+      </c>
+      <c r="E8" s="29" t="s">
+        <v>176</v>
+      </c>
+      <c r="F8" s="28">
+        <v>2017.0</v>
+      </c>
+      <c r="G8" s="28">
+        <v>2018.0</v>
+      </c>
+      <c r="H8" s="28">
+        <v>18686.0</v>
+      </c>
+      <c r="I8" s="30" t="s">
+        <v>177</v>
+      </c>
+      <c r="J8" s="30" t="s">
+        <v>178</v>
+      </c>
+      <c r="K8" s="28">
+        <v>289.0</v>
+      </c>
+      <c r="L8" s="30" t="s">
+        <v>179</v>
+      </c>
+      <c r="M8" s="28">
+        <v>65.5</v>
+      </c>
+      <c r="N8" s="28">
+        <v>40.996</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="29" t="s">
+        <v>180</v>
+      </c>
+      <c r="B9" s="30" t="s">
+        <v>79</v>
+      </c>
+      <c r="C9" s="28">
+        <v>1.0</v>
+      </c>
+      <c r="D9" s="28">
+        <v>0.5</v>
+      </c>
+      <c r="E9" s="29" t="s">
+        <v>181</v>
+      </c>
+      <c r="F9" s="28">
+        <v>2017.0</v>
+      </c>
+      <c r="G9" s="28">
+        <v>2018.0</v>
+      </c>
+      <c r="H9" s="28">
+        <v>87604.0</v>
+      </c>
+      <c r="I9" s="30" t="s">
+        <v>182</v>
+      </c>
+      <c r="J9" s="30" t="s">
+        <v>183</v>
+      </c>
+      <c r="K9" s="28">
+        <v>259.0</v>
+      </c>
+      <c r="L9" s="30" t="s">
+        <v>184</v>
+      </c>
+      <c r="M9" s="28">
+        <v>-50.105</v>
+      </c>
+      <c r="N9" s="28">
+        <v>-21.917</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="29" t="s">
+        <v>185</v>
+      </c>
+      <c r="B10" s="30" t="s">
         <v>104</v>
       </c>
-      <c r="F5" s="25">
-        <v>2017.0</v>
-      </c>
-      <c r="G5" s="25">
-        <v>2019.0</v>
-      </c>
-      <c r="H5" s="25">
-        <v>80936.0</v>
-      </c>
-      <c r="I5" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="J5" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="K5" s="25">
-        <v>569.0</v>
-      </c>
-      <c r="L5" s="25" t="s">
-        <v>101</v>
-      </c>
-      <c r="M5" s="25">
-        <v>11.087</v>
-      </c>
-      <c r="N5" s="25">
-        <v>53.882</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="24" t="s">
-        <v>96</v>
-      </c>
-      <c r="B6" s="25" t="s">
-        <v>97</v>
-      </c>
-      <c r="C6" s="25">
+      <c r="C10" s="28">
+        <v>2.0</v>
+      </c>
+      <c r="D10" s="28">
         <v>1.0</v>
       </c>
-      <c r="D6" s="25">
-        <v>0.25</v>
-      </c>
-      <c r="E6" s="24" t="s">
-        <v>105</v>
-      </c>
-      <c r="F6" s="25">
-        <v>2017.0</v>
-      </c>
-      <c r="G6" s="25">
-        <v>2019.0</v>
-      </c>
-      <c r="H6" s="25">
-        <v>80936.0</v>
-      </c>
-      <c r="I6" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="J6" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="K6" s="25">
-        <v>569.0</v>
-      </c>
-      <c r="L6" s="25" t="s">
-        <v>101</v>
-      </c>
-      <c r="M6" s="25">
-        <v>11.087</v>
-      </c>
-      <c r="N6" s="25">
-        <v>53.882</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="24" t="s">
-        <v>96</v>
-      </c>
-      <c r="B7" s="25" t="s">
-        <v>97</v>
-      </c>
-      <c r="C7" s="25">
+      <c r="E10" s="29" t="s">
+        <v>186</v>
+      </c>
+      <c r="F10" s="28">
+        <v>2018.0</v>
+      </c>
+      <c r="G10" s="28">
+        <v>2018.0</v>
+      </c>
+      <c r="H10" s="28">
+        <v>142608.0</v>
+      </c>
+      <c r="I10" s="30" t="s">
+        <v>187</v>
+      </c>
+      <c r="J10" s="30" t="s">
+        <v>188</v>
+      </c>
+      <c r="K10" s="28">
+        <v>277.0</v>
+      </c>
+      <c r="L10" s="30" t="s">
+        <v>189</v>
+      </c>
+      <c r="M10" s="28">
+        <v>144.5</v>
+      </c>
+      <c r="N10" s="28">
+        <v>-33.5</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="29" t="s">
+        <v>190</v>
+      </c>
+      <c r="B11" s="30" t="s">
+        <v>104</v>
+      </c>
+      <c r="C11" s="28">
+        <v>2.0</v>
+      </c>
+      <c r="D11" s="28">
+        <v>1.5</v>
+      </c>
+      <c r="E11" s="29" t="s">
+        <v>191</v>
+      </c>
+      <c r="F11" s="28">
+        <v>2018.0</v>
+      </c>
+      <c r="G11" s="28">
+        <v>2018.0</v>
+      </c>
+      <c r="H11" s="28">
+        <v>68692.0</v>
+      </c>
+      <c r="I11" s="30" t="s">
+        <v>192</v>
+      </c>
+      <c r="J11" s="30" t="s">
+        <v>193</v>
+      </c>
+      <c r="K11" s="28">
+        <v>177.0</v>
+      </c>
+      <c r="L11" s="30" t="s">
+        <v>194</v>
+      </c>
+      <c r="M11" s="28">
+        <v>46.464</v>
+      </c>
+      <c r="N11" s="28">
+        <v>-19.498</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="27" t="s">
+        <v>195</v>
+      </c>
+      <c r="B12" s="28" t="s">
+        <v>79</v>
+      </c>
+      <c r="C12" s="28">
         <v>1.0</v>
       </c>
-      <c r="D7" s="25">
-        <v>0.25</v>
-      </c>
-      <c r="E7" s="24" t="s">
-        <v>106</v>
-      </c>
-      <c r="F7" s="25">
-        <v>2017.0</v>
-      </c>
-      <c r="G7" s="25">
-        <v>2019.0</v>
-      </c>
-      <c r="H7" s="25">
-        <v>80936.0</v>
-      </c>
-      <c r="I7" s="25" t="s">
-        <v>99</v>
-      </c>
-      <c r="J7" s="25" t="s">
-        <v>100</v>
-      </c>
-      <c r="K7" s="25">
-        <v>569.0</v>
-      </c>
-      <c r="L7" s="25" t="s">
-        <v>101</v>
-      </c>
-      <c r="M7" s="25">
-        <v>11.087</v>
-      </c>
-      <c r="N7" s="25">
-        <v>53.882</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="26" t="s">
-        <v>107</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="C8" s="25">
-        <v>1.0</v>
-      </c>
-      <c r="D8" s="25">
+      <c r="D12" s="28">
         <v>0.75</v>
       </c>
-      <c r="E8" s="26" t="s">
-        <v>108</v>
-      </c>
-      <c r="F8" s="25">
-        <v>2017.0</v>
-      </c>
-      <c r="G8" s="25">
+      <c r="E12" s="27" t="s">
+        <v>181</v>
+      </c>
+      <c r="F12" s="28">
         <v>2018.0</v>
       </c>
-      <c r="H8" s="25">
-        <v>18686.0</v>
-      </c>
-      <c r="I8" s="21" t="s">
-        <v>109</v>
-      </c>
-      <c r="J8" s="21" t="s">
-        <v>110</v>
-      </c>
-      <c r="K8" s="25">
-        <v>289.0</v>
-      </c>
-      <c r="L8" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="M8" s="25">
-        <v>65.5</v>
-      </c>
-      <c r="N8" s="25">
-        <v>40.996</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="26" t="s">
-        <v>112</v>
-      </c>
-      <c r="B9" s="21" t="s">
-        <v>97</v>
-      </c>
-      <c r="C9" s="25">
-        <v>1.0</v>
-      </c>
-      <c r="D9" s="25">
-        <v>0.5</v>
-      </c>
-      <c r="E9" s="26" t="s">
-        <v>113</v>
-      </c>
-      <c r="F9" s="25">
-        <v>2017.0</v>
-      </c>
-      <c r="G9" s="25">
+      <c r="G12" s="28">
         <v>2018.0</v>
       </c>
-      <c r="H9" s="25">
-        <v>87604.0</v>
-      </c>
-      <c r="I9" s="21" t="s">
-        <v>114</v>
-      </c>
-      <c r="J9" s="21" t="s">
-        <v>115</v>
-      </c>
-      <c r="K9" s="25">
-        <v>259.0</v>
-      </c>
-      <c r="L9" s="21" t="s">
-        <v>116</v>
-      </c>
-      <c r="M9" s="25">
-        <v>-50.105</v>
-      </c>
-      <c r="N9" s="25">
-        <v>-21.917</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="26" t="s">
-        <v>117</v>
-      </c>
-      <c r="B10" s="21" t="s">
-        <v>118</v>
-      </c>
-      <c r="C10" s="25">
-        <v>2.0</v>
-      </c>
-      <c r="D10" s="25">
-        <v>1.0</v>
-      </c>
-      <c r="E10" s="26" t="s">
-        <v>119</v>
-      </c>
-      <c r="F10" s="25">
-        <v>2018.0</v>
-      </c>
-      <c r="G10" s="25">
-        <v>2018.0</v>
-      </c>
-      <c r="H10" s="25">
-        <v>142608.0</v>
-      </c>
-      <c r="I10" s="21" t="s">
-        <v>120</v>
-      </c>
-      <c r="J10" s="21" t="s">
-        <v>121</v>
-      </c>
-      <c r="K10" s="25">
-        <v>277.0</v>
-      </c>
-      <c r="L10" s="21" t="s">
-        <v>122</v>
-      </c>
-      <c r="M10" s="25">
-        <v>144.5</v>
-      </c>
-      <c r="N10" s="25">
-        <v>-33.5</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="26" t="s">
-        <v>123</v>
-      </c>
-      <c r="B11" s="21" t="s">
-        <v>118</v>
-      </c>
-      <c r="C11" s="25">
-        <v>2.0</v>
-      </c>
-      <c r="D11" s="25">
-        <v>1.5</v>
-      </c>
-      <c r="E11" s="26" t="s">
-        <v>124</v>
-      </c>
-      <c r="F11" s="25">
-        <v>2018.0</v>
-      </c>
-      <c r="G11" s="25">
-        <v>2018.0</v>
-      </c>
-      <c r="H11" s="25">
-        <v>68692.0</v>
-      </c>
-      <c r="I11" s="21" t="s">
-        <v>125</v>
-      </c>
-      <c r="J11" s="21" t="s">
-        <v>126</v>
-      </c>
-      <c r="K11" s="25">
-        <v>177.0</v>
-      </c>
-      <c r="L11" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="M11" s="25">
-        <v>46.464</v>
-      </c>
-      <c r="N11" s="25">
-        <v>-19.498</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="24" t="s">
-        <v>128</v>
-      </c>
-      <c r="B12" s="25" t="s">
-        <v>97</v>
-      </c>
-      <c r="C12" s="25">
-        <v>1.0</v>
-      </c>
-      <c r="D12" s="25">
-        <v>0.75</v>
-      </c>
-      <c r="E12" s="24" t="s">
-        <v>113</v>
-      </c>
-      <c r="F12" s="25">
-        <v>2018.0</v>
-      </c>
-      <c r="G12" s="25">
-        <v>2018.0</v>
-      </c>
-      <c r="H12" s="25">
+      <c r="H12" s="28">
         <v>104035.0</v>
       </c>
-      <c r="I12" s="25" t="s">
-        <v>114</v>
-      </c>
-      <c r="J12" s="25" t="s">
-        <v>129</v>
-      </c>
-      <c r="K12" s="25">
+      <c r="I12" s="28" t="s">
+        <v>182</v>
+      </c>
+      <c r="J12" s="28" t="s">
+        <v>196</v>
+      </c>
+      <c r="K12" s="28">
         <v>224.0</v>
       </c>
-      <c r="L12" s="25" t="s">
-        <v>130</v>
-      </c>
-      <c r="M12" s="25">
+      <c r="L12" s="28" t="s">
+        <v>197</v>
+      </c>
+      <c r="M12" s="28">
         <v>-38.05</v>
       </c>
-      <c r="N12" s="25">
+      <c r="N12" s="28">
         <v>-9.451</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="27"/>
-      <c r="E13" s="27"/>
+      <c r="A13" s="31"/>
+      <c r="E13" s="31"/>
     </row>
     <row r="14">
-      <c r="A14" s="27"/>
-      <c r="E14" s="27"/>
+      <c r="A14" s="31"/>
+      <c r="E14" s="31"/>
     </row>
     <row r="15">
-      <c r="A15" s="27"/>
-      <c r="E15" s="27"/>
+      <c r="A15" s="31"/>
+      <c r="E15" s="31"/>
     </row>
     <row r="16">
-      <c r="A16" s="27"/>
-      <c r="E16" s="27"/>
+      <c r="A16" s="31"/>
+      <c r="E16" s="31"/>
     </row>
     <row r="17">
-      <c r="A17" s="27"/>
-      <c r="E17" s="27"/>
+      <c r="A17" s="31"/>
+      <c r="E17" s="31"/>
     </row>
     <row r="18">
-      <c r="A18" s="27"/>
-      <c r="E18" s="27"/>
+      <c r="A18" s="31"/>
+      <c r="E18" s="31"/>
     </row>
     <row r="19">
-      <c r="A19" s="27"/>
-      <c r="E19" s="27"/>
+      <c r="A19" s="31"/>
+      <c r="E19" s="31"/>
     </row>
     <row r="20">
-      <c r="A20" s="27"/>
-      <c r="E20" s="27"/>
+      <c r="A20" s="31"/>
+      <c r="E20" s="31"/>
     </row>
     <row r="21">
-      <c r="A21" s="27"/>
-      <c r="E21" s="27"/>
+      <c r="A21" s="31"/>
+      <c r="E21" s="31"/>
     </row>
     <row r="22">
-      <c r="A22" s="27"/>
-      <c r="E22" s="27"/>
+      <c r="A22" s="31"/>
+      <c r="E22" s="31"/>
     </row>
     <row r="23">
-      <c r="A23" s="27"/>
-      <c r="E23" s="27"/>
+      <c r="A23" s="31"/>
+      <c r="E23" s="31"/>
     </row>
     <row r="24">
-      <c r="A24" s="27"/>
-      <c r="E24" s="27"/>
+      <c r="A24" s="31"/>
+      <c r="E24" s="31"/>
     </row>
     <row r="25">
-      <c r="A25" s="27"/>
-      <c r="E25" s="27"/>
+      <c r="A25" s="31"/>
+      <c r="E25" s="31"/>
     </row>
     <row r="26">
-      <c r="A26" s="27"/>
-      <c r="E26" s="27"/>
+      <c r="A26" s="31"/>
+      <c r="E26" s="31"/>
     </row>
     <row r="27">
-      <c r="A27" s="27"/>
-      <c r="E27" s="27"/>
+      <c r="A27" s="31"/>
+      <c r="E27" s="31"/>
     </row>
     <row r="28">
-      <c r="A28" s="27"/>
-      <c r="E28" s="27"/>
+      <c r="A28" s="31"/>
+      <c r="E28" s="31"/>
     </row>
     <row r="29">
-      <c r="A29" s="27"/>
-      <c r="E29" s="27"/>
+      <c r="A29" s="31"/>
+      <c r="E29" s="31"/>
     </row>
     <row r="30">
-      <c r="A30" s="27"/>
-      <c r="E30" s="27"/>
+      <c r="A30" s="31"/>
+      <c r="E30" s="31"/>
     </row>
     <row r="31">
-      <c r="A31" s="27"/>
-      <c r="E31" s="27"/>
+      <c r="A31" s="31"/>
+      <c r="E31" s="31"/>
     </row>
     <row r="32">
-      <c r="A32" s="27"/>
-      <c r="E32" s="27"/>
+      <c r="A32" s="31"/>
+      <c r="E32" s="31"/>
     </row>
     <row r="33">
-      <c r="A33" s="27"/>
-      <c r="E33" s="27"/>
+      <c r="A33" s="31"/>
+      <c r="E33" s="31"/>
     </row>
     <row r="34">
-      <c r="A34" s="27"/>
-      <c r="E34" s="27"/>
+      <c r="A34" s="31"/>
+      <c r="E34" s="31"/>
     </row>
     <row r="35">
-      <c r="A35" s="27"/>
-      <c r="E35" s="27"/>
+      <c r="A35" s="31"/>
+      <c r="E35" s="31"/>
     </row>
     <row r="36">
-      <c r="A36" s="27"/>
-      <c r="E36" s="27"/>
+      <c r="A36" s="31"/>
+      <c r="E36" s="31"/>
     </row>
     <row r="37">
-      <c r="A37" s="27"/>
-      <c r="E37" s="27"/>
+      <c r="A37" s="31"/>
+      <c r="E37" s="31"/>
     </row>
     <row r="38">
-      <c r="A38" s="27"/>
-      <c r="E38" s="27"/>
+      <c r="A38" s="31"/>
+      <c r="E38" s="31"/>
     </row>
     <row r="39">
-      <c r="A39" s="27"/>
-      <c r="E39" s="27"/>
+      <c r="A39" s="31"/>
+      <c r="E39" s="31"/>
     </row>
     <row r="40">
-      <c r="A40" s="27"/>
-      <c r="E40" s="27"/>
+      <c r="A40" s="31"/>
+      <c r="E40" s="31"/>
     </row>
     <row r="41">
-      <c r="A41" s="27"/>
-      <c r="E41" s="27"/>
+      <c r="A41" s="31"/>
+      <c r="E41" s="31"/>
     </row>
     <row r="42">
-      <c r="A42" s="27"/>
-      <c r="E42" s="27"/>
+      <c r="A42" s="31"/>
+      <c r="E42" s="31"/>
     </row>
     <row r="43">
-      <c r="A43" s="27"/>
-      <c r="E43" s="27"/>
+      <c r="A43" s="31"/>
+      <c r="E43" s="31"/>
     </row>
     <row r="44">
-      <c r="A44" s="27"/>
-      <c r="E44" s="27"/>
+      <c r="A44" s="31"/>
+      <c r="E44" s="31"/>
     </row>
     <row r="45">
-      <c r="A45" s="27"/>
-      <c r="E45" s="27"/>
+      <c r="A45" s="31"/>
+      <c r="E45" s="31"/>
     </row>
     <row r="46">
-      <c r="A46" s="27"/>
-      <c r="E46" s="27"/>
+      <c r="A46" s="31"/>
+      <c r="E46" s="31"/>
     </row>
     <row r="47">
-      <c r="A47" s="27"/>
-      <c r="E47" s="27"/>
+      <c r="A47" s="31"/>
+      <c r="E47" s="31"/>
     </row>
     <row r="48">
-      <c r="A48" s="27"/>
-      <c r="E48" s="27"/>
+      <c r="A48" s="31"/>
+      <c r="E48" s="31"/>
     </row>
     <row r="49">
-      <c r="A49" s="27"/>
-      <c r="E49" s="27"/>
+      <c r="A49" s="31"/>
+      <c r="E49" s="31"/>
     </row>
     <row r="50">
-      <c r="A50" s="27"/>
-      <c r="E50" s="27"/>
+      <c r="A50" s="31"/>
+      <c r="E50" s="31"/>
     </row>
     <row r="51">
-      <c r="A51" s="27"/>
-      <c r="E51" s="27"/>
+      <c r="A51" s="31"/>
+      <c r="E51" s="31"/>
     </row>
     <row r="52">
-      <c r="A52" s="27"/>
-      <c r="E52" s="27"/>
+      <c r="A52" s="31"/>
+      <c r="E52" s="31"/>
     </row>
     <row r="53">
-      <c r="A53" s="27"/>
-      <c r="E53" s="27"/>
+      <c r="A53" s="31"/>
+      <c r="E53" s="31"/>
     </row>
     <row r="54">
-      <c r="A54" s="27"/>
-      <c r="E54" s="27"/>
+      <c r="A54" s="31"/>
+      <c r="E54" s="31"/>
     </row>
     <row r="55">
-      <c r="A55" s="27"/>
-      <c r="E55" s="27"/>
+      <c r="A55" s="31"/>
+      <c r="E55" s="31"/>
     </row>
     <row r="56">
-      <c r="A56" s="27"/>
-      <c r="E56" s="27"/>
+      <c r="A56" s="31"/>
+      <c r="E56" s="31"/>
     </row>
     <row r="57">
-      <c r="A57" s="27"/>
-      <c r="E57" s="27"/>
+      <c r="A57" s="31"/>
+      <c r="E57" s="31"/>
     </row>
     <row r="58">
-      <c r="A58" s="27"/>
-      <c r="E58" s="27"/>
+      <c r="A58" s="31"/>
+      <c r="E58" s="31"/>
     </row>
     <row r="59">
-      <c r="A59" s="27"/>
-      <c r="E59" s="27"/>
+      <c r="A59" s="31"/>
+      <c r="E59" s="31"/>
     </row>
     <row r="60">
-      <c r="A60" s="27"/>
-      <c r="E60" s="27"/>
+      <c r="A60" s="31"/>
+      <c r="E60" s="31"/>
     </row>
     <row r="61">
-      <c r="A61" s="27"/>
-      <c r="E61" s="27"/>
+      <c r="A61" s="31"/>
+      <c r="E61" s="31"/>
     </row>
     <row r="62">
-      <c r="A62" s="27"/>
-      <c r="E62" s="27"/>
+      <c r="A62" s="31"/>
+      <c r="E62" s="31"/>
     </row>
     <row r="63">
-      <c r="A63" s="27"/>
-      <c r="E63" s="27"/>
+      <c r="A63" s="31"/>
+      <c r="E63" s="31"/>
     </row>
     <row r="64">
-      <c r="A64" s="27"/>
-      <c r="E64" s="27"/>
+      <c r="A64" s="31"/>
+      <c r="E64" s="31"/>
     </row>
     <row r="65">
-      <c r="A65" s="27"/>
-      <c r="E65" s="27"/>
+      <c r="A65" s="31"/>
+      <c r="E65" s="31"/>
     </row>
     <row r="66">
-      <c r="A66" s="27"/>
-      <c r="E66" s="27"/>
+      <c r="A66" s="31"/>
+      <c r="E66" s="31"/>
     </row>
     <row r="67">
-      <c r="A67" s="27"/>
-      <c r="E67" s="27"/>
+      <c r="A67" s="31"/>
+      <c r="E67" s="31"/>
     </row>
     <row r="68">
-      <c r="A68" s="27"/>
-      <c r="E68" s="27"/>
+      <c r="A68" s="31"/>
+      <c r="E68" s="31"/>
     </row>
     <row r="69">
-      <c r="A69" s="27"/>
-      <c r="E69" s="27"/>
+      <c r="A69" s="31"/>
+      <c r="E69" s="31"/>
     </row>
     <row r="70">
-      <c r="A70" s="27"/>
-      <c r="E70" s="27"/>
+      <c r="A70" s="31"/>
+      <c r="E70" s="31"/>
     </row>
     <row r="71">
-      <c r="A71" s="27"/>
-      <c r="E71" s="27"/>
+      <c r="A71" s="31"/>
+      <c r="E71" s="31"/>
     </row>
     <row r="72">
-      <c r="A72" s="27"/>
-      <c r="E72" s="27"/>
+      <c r="A72" s="31"/>
+      <c r="E72" s="31"/>
     </row>
     <row r="73">
-      <c r="A73" s="27"/>
-      <c r="E73" s="27"/>
+      <c r="A73" s="31"/>
+      <c r="E73" s="31"/>
     </row>
     <row r="74">
-      <c r="A74" s="27"/>
-      <c r="E74" s="27"/>
+      <c r="A74" s="31"/>
+      <c r="E74" s="31"/>
     </row>
     <row r="75">
-      <c r="A75" s="27"/>
-      <c r="E75" s="27"/>
+      <c r="A75" s="31"/>
+      <c r="E75" s="31"/>
     </row>
     <row r="76">
-      <c r="A76" s="27"/>
-      <c r="E76" s="27"/>
+      <c r="A76" s="31"/>
+      <c r="E76" s="31"/>
     </row>
     <row r="77">
-      <c r="A77" s="27"/>
-      <c r="E77" s="27"/>
+      <c r="A77" s="31"/>
+      <c r="E77" s="31"/>
     </row>
     <row r="78">
-      <c r="A78" s="27"/>
-      <c r="E78" s="27"/>
+      <c r="A78" s="31"/>
+      <c r="E78" s="31"/>
     </row>
     <row r="79">
-      <c r="A79" s="27"/>
-      <c r="E79" s="27"/>
+      <c r="A79" s="31"/>
+      <c r="E79" s="31"/>
     </row>
     <row r="80">
-      <c r="A80" s="27"/>
-      <c r="E80" s="27"/>
+      <c r="A80" s="31"/>
+      <c r="E80" s="31"/>
     </row>
     <row r="81">
-      <c r="A81" s="27"/>
-      <c r="E81" s="27"/>
+      <c r="A81" s="31"/>
+      <c r="E81" s="31"/>
     </row>
     <row r="82">
-      <c r="A82" s="27"/>
-      <c r="E82" s="27"/>
+      <c r="A82" s="31"/>
+      <c r="E82" s="31"/>
     </row>
     <row r="83">
-      <c r="A83" s="27"/>
-      <c r="E83" s="27"/>
+      <c r="A83" s="31"/>
+      <c r="E83" s="31"/>
     </row>
     <row r="84">
-      <c r="A84" s="27"/>
-      <c r="E84" s="27"/>
+      <c r="A84" s="31"/>
+      <c r="E84" s="31"/>
     </row>
     <row r="85">
-      <c r="A85" s="27"/>
-      <c r="E85" s="27"/>
+      <c r="A85" s="31"/>
+      <c r="E85" s="31"/>
     </row>
     <row r="86">
-      <c r="A86" s="27"/>
-      <c r="E86" s="27"/>
+      <c r="A86" s="31"/>
+      <c r="E86" s="31"/>
     </row>
     <row r="87">
-      <c r="A87" s="27"/>
-      <c r="E87" s="27"/>
+      <c r="A87" s="31"/>
+      <c r="E87" s="31"/>
     </row>
     <row r="88">
-      <c r="A88" s="27"/>
-      <c r="E88" s="27"/>
+      <c r="A88" s="31"/>
+      <c r="E88" s="31"/>
     </row>
     <row r="89">
-      <c r="A89" s="27"/>
-      <c r="E89" s="27"/>
+      <c r="A89" s="31"/>
+      <c r="E89" s="31"/>
     </row>
     <row r="90">
-      <c r="A90" s="27"/>
-      <c r="E90" s="27"/>
+      <c r="A90" s="31"/>
+      <c r="E90" s="31"/>
     </row>
     <row r="91">
-      <c r="A91" s="27"/>
-      <c r="E91" s="27"/>
+      <c r="A91" s="31"/>
+      <c r="E91" s="31"/>
     </row>
     <row r="92">
-      <c r="A92" s="27"/>
-      <c r="E92" s="27"/>
+      <c r="A92" s="31"/>
+      <c r="E92" s="31"/>
     </row>
     <row r="93">
-      <c r="A93" s="27"/>
-      <c r="E93" s="27"/>
+      <c r="A93" s="31"/>
+      <c r="E93" s="31"/>
     </row>
     <row r="94">
-      <c r="A94" s="27"/>
-      <c r="E94" s="27"/>
+      <c r="A94" s="31"/>
+      <c r="E94" s="31"/>
     </row>
     <row r="95">
-      <c r="A95" s="27"/>
-      <c r="E95" s="27"/>
+      <c r="A95" s="31"/>
+      <c r="E95" s="31"/>
     </row>
     <row r="96">
-      <c r="A96" s="27"/>
-      <c r="E96" s="27"/>
+      <c r="A96" s="31"/>
+      <c r="E96" s="31"/>
     </row>
     <row r="97">
-      <c r="A97" s="27"/>
-      <c r="E97" s="27"/>
+      <c r="A97" s="31"/>
+      <c r="E97" s="31"/>
     </row>
     <row r="98">
-      <c r="A98" s="27"/>
-      <c r="E98" s="27"/>
+      <c r="A98" s="31"/>
+      <c r="E98" s="31"/>
     </row>
     <row r="99">
-      <c r="A99" s="27"/>
-      <c r="E99" s="27"/>
+      <c r="A99" s="31"/>
+      <c r="E99" s="31"/>
     </row>
     <row r="100">
-      <c r="A100" s="27"/>
-      <c r="E100" s="27"/>
+      <c r="A100" s="31"/>
+      <c r="E100" s="31"/>
     </row>
     <row r="101">
-      <c r="A101" s="27"/>
-      <c r="E101" s="27"/>
+      <c r="A101" s="31"/>
+      <c r="E101" s="31"/>
     </row>
     <row r="102">
-      <c r="A102" s="27"/>
-      <c r="E102" s="27"/>
+      <c r="A102" s="31"/>
+      <c r="E102" s="31"/>
     </row>
     <row r="103">
-      <c r="A103" s="27"/>
-      <c r="E103" s="27"/>
+      <c r="A103" s="31"/>
+      <c r="E103" s="31"/>
     </row>
     <row r="104">
-      <c r="A104" s="27"/>
-      <c r="E104" s="27"/>
+      <c r="A104" s="31"/>
+      <c r="E104" s="31"/>
     </row>
     <row r="105">
-      <c r="A105" s="27"/>
-      <c r="E105" s="27"/>
+      <c r="A105" s="31"/>
+      <c r="E105" s="31"/>
     </row>
     <row r="106">
-      <c r="A106" s="27"/>
-      <c r="E106" s="27"/>
+      <c r="A106" s="31"/>
+      <c r="E106" s="31"/>
     </row>
     <row r="107">
-      <c r="A107" s="27"/>
-      <c r="E107" s="27"/>
+      <c r="A107" s="31"/>
+      <c r="E107" s="31"/>
     </row>
     <row r="108">
-      <c r="A108" s="27"/>
-      <c r="E108" s="27"/>
+      <c r="A108" s="31"/>
+      <c r="E108" s="31"/>
     </row>
     <row r="109">
-      <c r="A109" s="27"/>
-      <c r="E109" s="27"/>
+      <c r="A109" s="31"/>
+      <c r="E109" s="31"/>
     </row>
     <row r="110">
-      <c r="A110" s="27"/>
-      <c r="E110" s="27"/>
+      <c r="A110" s="31"/>
+      <c r="E110" s="31"/>
     </row>
     <row r="111">
-      <c r="A111" s="27"/>
-      <c r="E111" s="27"/>
+      <c r="A111" s="31"/>
+      <c r="E111" s="31"/>
     </row>
     <row r="112">
-      <c r="A112" s="27"/>
-      <c r="E112" s="27"/>
+      <c r="A112" s="31"/>
+      <c r="E112" s="31"/>
     </row>
     <row r="113">
-      <c r="A113" s="27"/>
-      <c r="E113" s="27"/>
+      <c r="A113" s="31"/>
+      <c r="E113" s="31"/>
     </row>
     <row r="114">
-      <c r="A114" s="27"/>
-      <c r="E114" s="27"/>
+      <c r="A114" s="31"/>
+      <c r="E114" s="31"/>
     </row>
     <row r="115">
-      <c r="A115" s="27"/>
-      <c r="E115" s="27"/>
+      <c r="A115" s="31"/>
+      <c r="E115" s="31"/>
     </row>
     <row r="116">
-      <c r="A116" s="27"/>
-      <c r="E116" s="27"/>
+      <c r="A116" s="31"/>
+      <c r="E116" s="31"/>
     </row>
     <row r="117">
-      <c r="A117" s="27"/>
-      <c r="E117" s="27"/>
+      <c r="A117" s="31"/>
+      <c r="E117" s="31"/>
     </row>
     <row r="118">
-      <c r="A118" s="27"/>
-      <c r="E118" s="27"/>
+      <c r="A118" s="31"/>
+      <c r="E118" s="31"/>
     </row>
     <row r="119">
-      <c r="A119" s="27"/>
-      <c r="E119" s="27"/>
+      <c r="A119" s="31"/>
+      <c r="E119" s="31"/>
     </row>
     <row r="120">
-      <c r="A120" s="27"/>
-      <c r="E120" s="27"/>
+      <c r="A120" s="31"/>
+      <c r="E120" s="31"/>
     </row>
     <row r="121">
-      <c r="A121" s="27"/>
-      <c r="E121" s="27"/>
+      <c r="A121" s="31"/>
+      <c r="E121" s="31"/>
     </row>
     <row r="122">
-      <c r="A122" s="27"/>
-      <c r="E122" s="27"/>
+      <c r="A122" s="31"/>
+      <c r="E122" s="31"/>
     </row>
     <row r="123">
-      <c r="A123" s="27"/>
-      <c r="E123" s="27"/>
+      <c r="A123" s="31"/>
+      <c r="E123" s="31"/>
     </row>
     <row r="124">
-      <c r="A124" s="27"/>
-      <c r="E124" s="27"/>
+      <c r="A124" s="31"/>
+      <c r="E124" s="31"/>
     </row>
     <row r="125">
-      <c r="A125" s="27"/>
-      <c r="E125" s="27"/>
+      <c r="A125" s="31"/>
+      <c r="E125" s="31"/>
     </row>
     <row r="126">
-      <c r="A126" s="27"/>
-      <c r="E126" s="27"/>
+      <c r="A126" s="31"/>
+      <c r="E126" s="31"/>
     </row>
     <row r="127">
-      <c r="A127" s="27"/>
-      <c r="E127" s="27"/>
+      <c r="A127" s="31"/>
+      <c r="E127" s="31"/>
     </row>
     <row r="128">
-      <c r="A128" s="27"/>
-      <c r="E128" s="27"/>
+      <c r="A128" s="31"/>
+      <c r="E128" s="31"/>
     </row>
     <row r="129">
-      <c r="A129" s="27"/>
-      <c r="E129" s="27"/>
+      <c r="A129" s="31"/>
+      <c r="E129" s="31"/>
     </row>
     <row r="130">
-      <c r="A130" s="27"/>
-      <c r="E130" s="27"/>
+      <c r="A130" s="31"/>
+      <c r="E130" s="31"/>
     </row>
     <row r="131">
-      <c r="A131" s="27"/>
-      <c r="E131" s="27"/>
+      <c r="A131" s="31"/>
+      <c r="E131" s="31"/>
     </row>
     <row r="132">
-      <c r="A132" s="27"/>
-      <c r="E132" s="27"/>
+      <c r="A132" s="31"/>
+      <c r="E132" s="31"/>
     </row>
     <row r="133">
-      <c r="A133" s="27"/>
-      <c r="E133" s="27"/>
+      <c r="A133" s="31"/>
+      <c r="E133" s="31"/>
     </row>
     <row r="134">
-      <c r="A134" s="27"/>
-      <c r="E134" s="27"/>
+      <c r="A134" s="31"/>
+      <c r="E134" s="31"/>
     </row>
     <row r="135">
-      <c r="A135" s="27"/>
-      <c r="E135" s="27"/>
+      <c r="A135" s="31"/>
+      <c r="E135" s="31"/>
     </row>
     <row r="136">
-      <c r="A136" s="27"/>
-      <c r="E136" s="27"/>
+      <c r="A136" s="31"/>
+      <c r="E136" s="31"/>
     </row>
     <row r="137">
-      <c r="A137" s="27"/>
-      <c r="E137" s="27"/>
+      <c r="A137" s="31"/>
+      <c r="E137" s="31"/>
     </row>
     <row r="138">
-      <c r="A138" s="27"/>
-      <c r="E138" s="27"/>
+      <c r="A138" s="31"/>
+      <c r="E138" s="31"/>
     </row>
     <row r="139">
-      <c r="A139" s="27"/>
-      <c r="E139" s="27"/>
+      <c r="A139" s="31"/>
+      <c r="E139" s="31"/>
     </row>
     <row r="140">
-      <c r="A140" s="27"/>
-      <c r="E140" s="27"/>
+      <c r="A140" s="31"/>
+      <c r="E140" s="31"/>
     </row>
     <row r="141">
-      <c r="A141" s="27"/>
-      <c r="E141" s="27"/>
+      <c r="A141" s="31"/>
+      <c r="E141" s="31"/>
     </row>
     <row r="142">
-      <c r="A142" s="27"/>
-      <c r="E142" s="27"/>
+      <c r="A142" s="31"/>
+      <c r="E142" s="31"/>
     </row>
     <row r="143">
-      <c r="A143" s="27"/>
-      <c r="E143" s="27"/>
+      <c r="A143" s="31"/>
+      <c r="E143" s="31"/>
     </row>
     <row r="144">
-      <c r="A144" s="27"/>
-      <c r="E144" s="27"/>
+      <c r="A144" s="31"/>
+      <c r="E144" s="31"/>
     </row>
     <row r="145">
-      <c r="A145" s="27"/>
-      <c r="E145" s="27"/>
+      <c r="A145" s="31"/>
+      <c r="E145" s="31"/>
     </row>
     <row r="146">
-      <c r="A146" s="27"/>
-      <c r="E146" s="27"/>
+      <c r="A146" s="31"/>
+      <c r="E146" s="31"/>
     </row>
     <row r="147">
-      <c r="A147" s="27"/>
-      <c r="E147" s="27"/>
+      <c r="A147" s="31"/>
+      <c r="E147" s="31"/>
     </row>
     <row r="148">
-      <c r="A148" s="27"/>
-      <c r="E148" s="27"/>
+      <c r="A148" s="31"/>
+      <c r="E148" s="31"/>
     </row>
     <row r="149">
-      <c r="A149" s="27"/>
-      <c r="E149" s="27"/>
+      <c r="A149" s="31"/>
+      <c r="E149" s="31"/>
     </row>
     <row r="150">
-      <c r="A150" s="27"/>
-      <c r="E150" s="27"/>
+      <c r="A150" s="31"/>
+      <c r="E150" s="31"/>
     </row>
     <row r="151">
-      <c r="A151" s="27"/>
-      <c r="E151" s="27"/>
+      <c r="A151" s="31"/>
+      <c r="E151" s="31"/>
     </row>
     <row r="152">
-      <c r="A152" s="27"/>
-      <c r="E152" s="27"/>
+      <c r="A152" s="31"/>
+      <c r="E152" s="31"/>
     </row>
     <row r="153">
-      <c r="A153" s="27"/>
-      <c r="E153" s="27"/>
+      <c r="A153" s="31"/>
+      <c r="E153" s="31"/>
     </row>
     <row r="154">
-      <c r="A154" s="27"/>
-      <c r="E154" s="27"/>
+      <c r="A154" s="31"/>
+      <c r="E154" s="31"/>
     </row>
     <row r="155">
-      <c r="A155" s="27"/>
-      <c r="E155" s="27"/>
+      <c r="A155" s="31"/>
+      <c r="E155" s="31"/>
     </row>
     <row r="156">
-      <c r="A156" s="27"/>
-      <c r="E156" s="27"/>
+      <c r="A156" s="31"/>
+      <c r="E156" s="31"/>
     </row>
     <row r="157">
-      <c r="A157" s="27"/>
-      <c r="E157" s="27"/>
+      <c r="A157" s="31"/>
+      <c r="E157" s="31"/>
     </row>
     <row r="158">
-      <c r="A158" s="27"/>
-      <c r="E158" s="27"/>
+      <c r="A158" s="31"/>
+      <c r="E158" s="31"/>
     </row>
     <row r="159">
-      <c r="A159" s="27"/>
-      <c r="E159" s="27"/>
+      <c r="A159" s="31"/>
+      <c r="E159" s="31"/>
     </row>
     <row r="160">
-      <c r="A160" s="27"/>
-      <c r="E160" s="27"/>
+      <c r="A160" s="31"/>
+      <c r="E160" s="31"/>
     </row>
     <row r="161">
-      <c r="A161" s="27"/>
-      <c r="E161" s="27"/>
+      <c r="A161" s="31"/>
+      <c r="E161" s="31"/>
     </row>
     <row r="162">
-      <c r="A162" s="27"/>
-      <c r="E162" s="27"/>
+      <c r="A162" s="31"/>
+      <c r="E162" s="31"/>
     </row>
     <row r="163">
-      <c r="A163" s="27"/>
-      <c r="E163" s="27"/>
+      <c r="A163" s="31"/>
+      <c r="E163" s="31"/>
     </row>
     <row r="164">
-      <c r="A164" s="27"/>
-      <c r="E164" s="27"/>
+      <c r="A164" s="31"/>
+      <c r="E164" s="31"/>
     </row>
     <row r="165">
-      <c r="A165" s="27"/>
-      <c r="E165" s="27"/>
+      <c r="A165" s="31"/>
+      <c r="E165" s="31"/>
     </row>
     <row r="166">
-      <c r="A166" s="27"/>
-      <c r="E166" s="27"/>
+      <c r="A166" s="31"/>
+      <c r="E166" s="31"/>
     </row>
     <row r="167">
-      <c r="A167" s="27"/>
-      <c r="E167" s="27"/>
+      <c r="A167" s="31"/>
+      <c r="E167" s="31"/>
     </row>
     <row r="168">
-      <c r="A168" s="27"/>
-      <c r="E168" s="27"/>
+      <c r="A168" s="31"/>
+      <c r="E168" s="31"/>
     </row>
     <row r="169">
-      <c r="A169" s="27"/>
-      <c r="E169" s="27"/>
+      <c r="A169" s="31"/>
+      <c r="E169" s="31"/>
     </row>
     <row r="170">
-      <c r="A170" s="27"/>
-      <c r="E170" s="27"/>
+      <c r="A170" s="31"/>
+      <c r="E170" s="31"/>
     </row>
     <row r="171">
-      <c r="A171" s="27"/>
-      <c r="E171" s="27"/>
+      <c r="A171" s="31"/>
+      <c r="E171" s="31"/>
     </row>
     <row r="172">
-      <c r="A172" s="27"/>
-      <c r="E172" s="27"/>
+      <c r="A172" s="31"/>
+      <c r="E172" s="31"/>
     </row>
     <row r="173">
-      <c r="A173" s="27"/>
-      <c r="E173" s="27"/>
+      <c r="A173" s="31"/>
+      <c r="E173" s="31"/>
     </row>
     <row r="174">
-      <c r="A174" s="27"/>
-      <c r="E174" s="27"/>
+      <c r="A174" s="31"/>
+      <c r="E174" s="31"/>
     </row>
     <row r="175">
-      <c r="A175" s="27"/>
-      <c r="E175" s="27"/>
+      <c r="A175" s="31"/>
+      <c r="E175" s="31"/>
     </row>
     <row r="176">
-      <c r="A176" s="27"/>
-      <c r="E176" s="27"/>
+      <c r="A176" s="31"/>
+      <c r="E176" s="31"/>
     </row>
     <row r="177">
-      <c r="A177" s="27"/>
-      <c r="E177" s="27"/>
+      <c r="A177" s="31"/>
+      <c r="E177" s="31"/>
     </row>
     <row r="178">
-      <c r="A178" s="27"/>
-      <c r="E178" s="27"/>
+      <c r="A178" s="31"/>
+      <c r="E178" s="31"/>
     </row>
     <row r="179">
-      <c r="A179" s="27"/>
-      <c r="E179" s="27"/>
+      <c r="A179" s="31"/>
+      <c r="E179" s="31"/>
     </row>
     <row r="180">
-      <c r="A180" s="27"/>
-      <c r="E180" s="27"/>
+      <c r="A180" s="31"/>
+      <c r="E180" s="31"/>
     </row>
     <row r="181">
-      <c r="A181" s="27"/>
-      <c r="E181" s="27"/>
+      <c r="A181" s="31"/>
+      <c r="E181" s="31"/>
     </row>
     <row r="182">
-      <c r="A182" s="27"/>
-      <c r="E182" s="27"/>
+      <c r="A182" s="31"/>
+      <c r="E182" s="31"/>
     </row>
     <row r="183">
-      <c r="A183" s="27"/>
-      <c r="E183" s="27"/>
+      <c r="A183" s="31"/>
+      <c r="E183" s="31"/>
     </row>
     <row r="184">
-      <c r="A184" s="27"/>
-      <c r="E184" s="27"/>
+      <c r="A184" s="31"/>
+      <c r="E184" s="31"/>
     </row>
     <row r="185">
-      <c r="A185" s="27"/>
-      <c r="E185" s="27"/>
+      <c r="A185" s="31"/>
+      <c r="E185" s="31"/>
     </row>
     <row r="186">
-      <c r="A186" s="27"/>
-      <c r="E186" s="27"/>
+      <c r="A186" s="31"/>
+      <c r="E186" s="31"/>
     </row>
     <row r="187">
-      <c r="A187" s="27"/>
-      <c r="E187" s="27"/>
+      <c r="A187" s="31"/>
+      <c r="E187" s="31"/>
     </row>
     <row r="188">
-      <c r="A188" s="27"/>
-      <c r="E188" s="27"/>
+      <c r="A188" s="31"/>
+      <c r="E188" s="31"/>
     </row>
     <row r="189">
-      <c r="A189" s="27"/>
-      <c r="E189" s="27"/>
+      <c r="A189" s="31"/>
+      <c r="E189" s="31"/>
     </row>
     <row r="190">
-      <c r="A190" s="27"/>
-      <c r="E190" s="27"/>
+      <c r="A190" s="31"/>
+      <c r="E190" s="31"/>
     </row>
     <row r="191">
-      <c r="A191" s="27"/>
-      <c r="E191" s="27"/>
+      <c r="A191" s="31"/>
+      <c r="E191" s="31"/>
     </row>
     <row r="192">
-      <c r="A192" s="27"/>
-      <c r="E192" s="27"/>
+      <c r="A192" s="31"/>
+      <c r="E192" s="31"/>
     </row>
     <row r="193">
-      <c r="A193" s="27"/>
-      <c r="E193" s="27"/>
+      <c r="A193" s="31"/>
+      <c r="E193" s="31"/>
     </row>
     <row r="194">
-      <c r="A194" s="27"/>
-      <c r="E194" s="27"/>
+      <c r="A194" s="31"/>
+      <c r="E194" s="31"/>
     </row>
     <row r="195">
-      <c r="A195" s="27"/>
-      <c r="E195" s="27"/>
+      <c r="A195" s="31"/>
+      <c r="E195" s="31"/>
     </row>
     <row r="196">
-      <c r="A196" s="27"/>
-      <c r="E196" s="27"/>
+      <c r="A196" s="31"/>
+      <c r="E196" s="31"/>
     </row>
     <row r="197">
-      <c r="A197" s="27"/>
-      <c r="E197" s="27"/>
+      <c r="A197" s="31"/>
+      <c r="E197" s="31"/>
     </row>
     <row r="198">
-      <c r="A198" s="27"/>
-      <c r="E198" s="27"/>
+      <c r="A198" s="31"/>
+      <c r="E198" s="31"/>
     </row>
     <row r="199">
-      <c r="A199" s="27"/>
-      <c r="E199" s="27"/>
+      <c r="A199" s="31"/>
+      <c r="E199" s="31"/>
     </row>
     <row r="200">
-      <c r="A200" s="27"/>
-      <c r="E200" s="27"/>
+      <c r="A200" s="31"/>
+      <c r="E200" s="31"/>
     </row>
     <row r="201">
-      <c r="A201" s="27"/>
-      <c r="E201" s="27"/>
+      <c r="A201" s="31"/>
+      <c r="E201" s="31"/>
     </row>
     <row r="202">
-      <c r="A202" s="27"/>
-      <c r="E202" s="27"/>
+      <c r="A202" s="31"/>
+      <c r="E202" s="31"/>
     </row>
     <row r="203">
-      <c r="A203" s="27"/>
-      <c r="E203" s="27"/>
+      <c r="A203" s="31"/>
+      <c r="E203" s="31"/>
     </row>
     <row r="204">
-      <c r="A204" s="27"/>
-      <c r="E204" s="27"/>
+      <c r="A204" s="31"/>
+      <c r="E204" s="31"/>
     </row>
     <row r="205">
-      <c r="A205" s="27"/>
-      <c r="E205" s="27"/>
+      <c r="A205" s="31"/>
+      <c r="E205" s="31"/>
     </row>
     <row r="206">
-      <c r="A206" s="27"/>
-      <c r="E206" s="27"/>
+      <c r="A206" s="31"/>
+      <c r="E206" s="31"/>
     </row>
     <row r="207">
-      <c r="A207" s="27"/>
-      <c r="E207" s="27"/>
+      <c r="A207" s="31"/>
+      <c r="E207" s="31"/>
     </row>
     <row r="208">
-      <c r="A208" s="27"/>
-      <c r="E208" s="27"/>
+      <c r="A208" s="31"/>
+      <c r="E208" s="31"/>
     </row>
     <row r="209">
-      <c r="A209" s="27"/>
-      <c r="E209" s="27"/>
+      <c r="A209" s="31"/>
+      <c r="E209" s="31"/>
     </row>
     <row r="210">
-      <c r="A210" s="27"/>
-      <c r="E210" s="27"/>
+      <c r="A210" s="31"/>
+      <c r="E210" s="31"/>
     </row>
     <row r="211">
-      <c r="A211" s="27"/>
-      <c r="E211" s="27"/>
+      <c r="A211" s="31"/>
+      <c r="E211" s="31"/>
     </row>
     <row r="212">
-      <c r="A212" s="27"/>
-      <c r="E212" s="27"/>
+      <c r="A212" s="31"/>
+      <c r="E212" s="31"/>
     </row>
     <row r="213">
-      <c r="A213" s="27"/>
-      <c r="E213" s="27"/>
+      <c r="A213" s="31"/>
+      <c r="E213" s="31"/>
     </row>
     <row r="214">
-      <c r="A214" s="27"/>
-      <c r="E214" s="27"/>
+      <c r="A214" s="31"/>
+      <c r="E214" s="31"/>
     </row>
     <row r="215">
-      <c r="A215" s="27"/>
-      <c r="E215" s="27"/>
+      <c r="A215" s="31"/>
+      <c r="E215" s="31"/>
     </row>
     <row r="216">
-      <c r="A216" s="27"/>
-      <c r="E216" s="27"/>
+      <c r="A216" s="31"/>
+      <c r="E216" s="31"/>
     </row>
     <row r="217">
-      <c r="A217" s="27"/>
-      <c r="E217" s="27"/>
+      <c r="A217" s="31"/>
+      <c r="E217" s="31"/>
     </row>
     <row r="218">
-      <c r="A218" s="27"/>
-      <c r="E218" s="27"/>
+      <c r="A218" s="31"/>
+      <c r="E218" s="31"/>
     </row>
     <row r="219">
-      <c r="A219" s="27"/>
-      <c r="E219" s="27"/>
+      <c r="A219" s="31"/>
+      <c r="E219" s="31"/>
     </row>
     <row r="220">
-      <c r="A220" s="27"/>
-      <c r="E220" s="27"/>
+      <c r="A220" s="31"/>
+      <c r="E220" s="31"/>
     </row>
     <row r="221">
-      <c r="A221" s="27"/>
-      <c r="E221" s="27"/>
+      <c r="A221" s="31"/>
+      <c r="E221" s="31"/>
     </row>
     <row r="222">
-      <c r="A222" s="27"/>
-      <c r="E222" s="27"/>
+      <c r="A222" s="31"/>
+      <c r="E222" s="31"/>
     </row>
     <row r="223">
-      <c r="A223" s="27"/>
-      <c r="E223" s="27"/>
+      <c r="A223" s="31"/>
+      <c r="E223" s="31"/>
     </row>
     <row r="224">
-      <c r="A224" s="27"/>
-      <c r="E224" s="27"/>
+      <c r="A224" s="31"/>
+      <c r="E224" s="31"/>
     </row>
     <row r="225">
-      <c r="A225" s="27"/>
-      <c r="E225" s="27"/>
+      <c r="A225" s="31"/>
+      <c r="E225" s="31"/>
     </row>
     <row r="226">
-      <c r="A226" s="27"/>
-      <c r="E226" s="27"/>
+      <c r="A226" s="31"/>
+      <c r="E226" s="31"/>
     </row>
     <row r="227">
-      <c r="A227" s="27"/>
-      <c r="E227" s="27"/>
+      <c r="A227" s="31"/>
+      <c r="E227" s="31"/>
     </row>
     <row r="228">
-      <c r="A228" s="27"/>
-      <c r="E228" s="27"/>
+      <c r="A228" s="31"/>
+      <c r="E228" s="31"/>
     </row>
     <row r="229">
-      <c r="A229" s="27"/>
-      <c r="E229" s="27"/>
+      <c r="A229" s="31"/>
+      <c r="E229" s="31"/>
     </row>
     <row r="230">
-      <c r="A230" s="27"/>
-      <c r="E230" s="27"/>
+      <c r="A230" s="31"/>
+      <c r="E230" s="31"/>
     </row>
     <row r="231">
-      <c r="A231" s="27"/>
-      <c r="E231" s="27"/>
+      <c r="A231" s="31"/>
+      <c r="E231" s="31"/>
     </row>
     <row r="232">
-      <c r="A232" s="27"/>
-      <c r="E232" s="27"/>
+      <c r="A232" s="31"/>
+      <c r="E232" s="31"/>
     </row>
     <row r="233">
-      <c r="A233" s="27"/>
-      <c r="E233" s="27"/>
+      <c r="A233" s="31"/>
+      <c r="E233" s="31"/>
     </row>
     <row r="234">
-      <c r="A234" s="27"/>
-      <c r="E234" s="27"/>
+      <c r="A234" s="31"/>
+      <c r="E234" s="31"/>
     </row>
     <row r="235">
-      <c r="A235" s="27"/>
-      <c r="E235" s="27"/>
+      <c r="A235" s="31"/>
+      <c r="E235" s="31"/>
     </row>
     <row r="236">
-      <c r="A236" s="27"/>
-      <c r="E236" s="27"/>
+      <c r="A236" s="31"/>
+      <c r="E236" s="31"/>
     </row>
     <row r="237">
-      <c r="A237" s="27"/>
-      <c r="E237" s="27"/>
+      <c r="A237" s="31"/>
+      <c r="E237" s="31"/>
     </row>
     <row r="238">
-      <c r="A238" s="27"/>
-      <c r="E238" s="27"/>
+      <c r="A238" s="31"/>
+      <c r="E238" s="31"/>
     </row>
     <row r="239">
-      <c r="A239" s="27"/>
-      <c r="E239" s="27"/>
+      <c r="A239" s="31"/>
+      <c r="E239" s="31"/>
     </row>
     <row r="240">
-      <c r="A240" s="27"/>
-      <c r="E240" s="27"/>
+      <c r="A240" s="31"/>
+      <c r="E240" s="31"/>
     </row>
     <row r="241">
-      <c r="A241" s="27"/>
-      <c r="E241" s="27"/>
+      <c r="A241" s="31"/>
+      <c r="E241" s="31"/>
     </row>
     <row r="242">
-      <c r="A242" s="27"/>
-      <c r="E242" s="27"/>
+      <c r="A242" s="31"/>
+      <c r="E242" s="31"/>
     </row>
     <row r="243">
-      <c r="A243" s="27"/>
-      <c r="E243" s="27"/>
+      <c r="A243" s="31"/>
+      <c r="E243" s="31"/>
     </row>
     <row r="244">
-      <c r="A244" s="27"/>
-      <c r="E244" s="27"/>
+      <c r="A244" s="31"/>
+      <c r="E244" s="31"/>
     </row>
     <row r="245">
-      <c r="A245" s="27"/>
-      <c r="E245" s="27"/>
+      <c r="A245" s="31"/>
+      <c r="E245" s="31"/>
     </row>
     <row r="246">
-      <c r="A246" s="27"/>
-      <c r="E246" s="27"/>
+      <c r="A246" s="31"/>
+      <c r="E246" s="31"/>
     </row>
     <row r="247">
-      <c r="A247" s="27"/>
-      <c r="E247" s="27"/>
+      <c r="A247" s="31"/>
+      <c r="E247" s="31"/>
     </row>
     <row r="248">
-      <c r="A248" s="27"/>
-      <c r="E248" s="27"/>
+      <c r="A248" s="31"/>
+      <c r="E248" s="31"/>
     </row>
     <row r="249">
-      <c r="A249" s="27"/>
-      <c r="E249" s="27"/>
+      <c r="A249" s="31"/>
+      <c r="E249" s="31"/>
     </row>
     <row r="250">
-      <c r="A250" s="27"/>
-      <c r="E250" s="27"/>
+      <c r="A250" s="31"/>
+      <c r="E250" s="31"/>
     </row>
   </sheetData>
   <drawing r:id="rId1"/>

</xml_diff>

<commit_message>
Revision del entregable D01 - earthquakes
</commit_message>
<xml_diff>
--- a/SOS2526-19-Propuesta.xlsx
+++ b/SOS2526-19-Propuesta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\javim\Desktop\CARRERA\3º DE CARRERA\2O CUATRIMESTRE\SOS\SOS2526-19\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC7EF1C1-37BD-48BE-A09F-E82AA5193292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95FF86B3-FE8B-4B0A-B2B9-B820A706BB93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="220">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="218">
   <si>
     <t>Nombre / enlace repositorio Github</t>
   </si>
@@ -331,9 +331,6 @@
     <t>4.9M</t>
   </si>
   <si>
-    <t>0 Km</t>
-  </si>
-  <si>
     <t>440000 people within 100km</t>
   </si>
   <si>
@@ -449,9 +446,6 @@
   </si>
   <si>
     <t>6.5M</t>
-  </si>
-  <si>
-    <t>10 Km</t>
   </si>
   <si>
     <t>3 thousand in MMI VI</t>
@@ -1056,9 +1050,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:H9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2" spans="2:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>0</v>
       </c>
@@ -1069,12 +1063,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="3" spans="2:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B3" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="2:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B4" t="s">
         <v>4</v>
       </c>
@@ -1086,14 +1080,14 @@
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
     </row>
-    <row r="5" spans="2:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:8" x14ac:dyDescent="0.25">
       <c r="C5" s="1"/>
       <c r="D5" s="1"/>
       <c r="E5" s="1"/>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
     </row>
-    <row r="6" spans="2:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B6" t="s">
         <v>6</v>
       </c>
@@ -1116,7 +1110,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="2:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B7" t="s">
         <v>13</v>
       </c>
@@ -1139,7 +1133,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="2:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B8" t="s">
         <v>19</v>
       </c>
@@ -1162,7 +1156,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="2:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B9" t="s">
         <v>25</v>
       </c>
@@ -1205,9 +1199,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Z11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>30</v>
       </c>
@@ -1287,7 +1281,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="2" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>56</v>
       </c>
@@ -1319,7 +1313,7 @@
         <v>0.27819484500000002</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>56</v>
       </c>
@@ -1351,7 +1345,7 @@
         <v>0.27001029300000001</v>
       </c>
     </row>
-    <row r="4" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>57</v>
       </c>
@@ -1383,7 +1377,7 @@
         <v>0.25693634199999998</v>
       </c>
     </row>
-    <row r="5" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>56</v>
       </c>
@@ -1415,7 +1409,7 @@
         <v>0.25945362399999999</v>
       </c>
     </row>
-    <row r="6" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>56</v>
       </c>
@@ -1447,7 +1441,7 @@
         <v>0.26945251199999998</v>
       </c>
     </row>
-    <row r="7" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>58</v>
       </c>
@@ -1479,7 +1473,7 @@
         <v>0.14376196299999999</v>
       </c>
     </row>
-    <row r="8" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>58</v>
       </c>
@@ -1511,7 +1505,7 @@
         <v>0.15634134399999999</v>
       </c>
     </row>
-    <row r="9" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>60</v>
       </c>
@@ -1543,7 +1537,7 @@
         <v>0.166525215</v>
       </c>
     </row>
-    <row r="10" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>61</v>
       </c>
@@ -1575,7 +1569,7 @@
         <v>0.139507085</v>
       </c>
     </row>
-    <row r="11" spans="1:26" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>62</v>
       </c>
@@ -1618,7 +1612,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:U12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="15.75" customWidth="1"/>
     <col min="2" max="2" width="40.125" customWidth="1"/>
@@ -1632,7 +1626,7 @@
     <col min="19" max="19" width="30.625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>63</v>
       </c>
@@ -1697,7 +1691,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="2" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>83</v>
       </c>
@@ -1759,7 +1753,7 @@
         <v>1320000</v>
       </c>
     </row>
-    <row r="3" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>95</v>
       </c>
@@ -1811,16 +1805,16 @@
       <c r="Q3" t="s">
         <v>101</v>
       </c>
-      <c r="R3" t="s">
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3" t="s">
         <v>102</v>
       </c>
-      <c r="S3" t="s">
+    </row>
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row r="4" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>104</v>
       </c>
       <c r="B4" t="s">
         <v>96</v>
@@ -1829,7 +1823,7 @@
         <v>96</v>
       </c>
       <c r="D4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E4" t="s">
         <v>86</v>
@@ -1856,7 +1850,7 @@
         <v>5.3</v>
       </c>
       <c r="M4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="N4" t="s">
         <v>90</v>
@@ -1868,27 +1862,27 @@
         <v>92</v>
       </c>
       <c r="Q4" t="s">
+        <v>106</v>
+      </c>
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4" t="s">
         <v>107</v>
       </c>
-      <c r="R4" t="s">
-        <v>102</v>
-      </c>
-      <c r="S4" t="s">
+    </row>
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>108</v>
       </c>
-    </row>
-    <row r="5" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="B5" t="s">
         <v>109</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
+        <v>109</v>
+      </c>
+      <c r="D5" t="s">
         <v>110</v>
-      </c>
-      <c r="C5" t="s">
-        <v>110</v>
-      </c>
-      <c r="D5" t="s">
-        <v>111</v>
       </c>
       <c r="E5" t="s">
         <v>86</v>
@@ -1906,63 +1900,63 @@
         <v>62</v>
       </c>
       <c r="J5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="K5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="L5">
         <v>5.5</v>
       </c>
       <c r="M5" t="s">
+        <v>112</v>
+      </c>
+      <c r="N5" t="s">
         <v>113</v>
       </c>
-      <c r="N5" t="s">
+      <c r="O5" t="s">
         <v>114</v>
-      </c>
-      <c r="O5" t="s">
-        <v>115</v>
       </c>
       <c r="P5" t="s">
         <v>92</v>
       </c>
       <c r="Q5" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="R5">
         <v>10</v>
       </c>
       <c r="S5" t="s">
+        <v>116</v>
+      </c>
+      <c r="T5" t="s">
         <v>117</v>
-      </c>
-      <c r="T5" t="s">
-        <v>118</v>
       </c>
       <c r="U5">
         <v>30000</v>
       </c>
     </row>
-    <row r="6" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>118</v>
+      </c>
+      <c r="B6" t="s">
         <v>119</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
+        <v>119</v>
+      </c>
+      <c r="D6" t="s">
         <v>120</v>
       </c>
-      <c r="C6" t="s">
-        <v>120</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="E6" t="s">
         <v>121</v>
-      </c>
-      <c r="E6" t="s">
-        <v>122</v>
       </c>
       <c r="F6">
         <v>2</v>
       </c>
       <c r="G6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H6">
         <v>1.5</v>
@@ -1971,63 +1965,63 @@
         <v>61</v>
       </c>
       <c r="J6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="K6" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="L6">
         <v>7.6</v>
       </c>
       <c r="M6" t="s">
+        <v>123</v>
+      </c>
+      <c r="N6" t="s">
+        <v>113</v>
+      </c>
+      <c r="O6" t="s">
         <v>124</v>
-      </c>
-      <c r="N6" t="s">
-        <v>114</v>
-      </c>
-      <c r="O6" t="s">
-        <v>125</v>
       </c>
       <c r="P6" t="s">
         <v>92</v>
       </c>
       <c r="Q6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="R6">
         <v>10</v>
       </c>
       <c r="S6" t="s">
+        <v>126</v>
+      </c>
+      <c r="T6" t="s">
         <v>127</v>
-      </c>
-      <c r="T6" t="s">
-        <v>128</v>
       </c>
       <c r="U6">
         <v>90000</v>
       </c>
     </row>
-    <row r="7" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>128</v>
+      </c>
+      <c r="B7" t="s">
         <v>129</v>
       </c>
-      <c r="B7" t="s">
+      <c r="C7" t="s">
+        <v>129</v>
+      </c>
+      <c r="D7" t="s">
         <v>130</v>
       </c>
-      <c r="C7" t="s">
-        <v>130</v>
-      </c>
-      <c r="D7" t="s">
-        <v>131</v>
-      </c>
       <c r="E7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="F7">
         <v>2</v>
       </c>
       <c r="G7" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="H7">
         <v>1.05</v>
@@ -2036,54 +2030,54 @@
         <v>60</v>
       </c>
       <c r="J7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="K7" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="L7">
         <v>7.9</v>
       </c>
       <c r="M7" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="N7" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="O7" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P7" t="s">
         <v>92</v>
       </c>
       <c r="Q7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="R7">
         <v>10</v>
       </c>
       <c r="S7" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="T7" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="U7">
         <v>1000</v>
       </c>
     </row>
-    <row r="8" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>135</v>
+      </c>
+      <c r="B8" t="s">
         <v>136</v>
       </c>
-      <c r="B8" t="s">
+      <c r="C8" t="s">
+        <v>136</v>
+      </c>
+      <c r="D8" t="s">
         <v>137</v>
-      </c>
-      <c r="C8" t="s">
-        <v>137</v>
-      </c>
-      <c r="D8" t="s">
-        <v>138</v>
       </c>
       <c r="E8" t="s">
         <v>86</v>
@@ -2098,7 +2092,7 @@
         <v>0.5</v>
       </c>
       <c r="I8" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="J8">
         <v>36737.517361111109</v>
@@ -2110,42 +2104,42 @@
         <v>6.5</v>
       </c>
       <c r="M8" t="s">
+        <v>138</v>
+      </c>
+      <c r="N8" t="s">
+        <v>113</v>
+      </c>
+      <c r="O8" t="s">
         <v>139</v>
-      </c>
-      <c r="N8" t="s">
-        <v>114</v>
-      </c>
-      <c r="O8" t="s">
-        <v>140</v>
       </c>
       <c r="P8" t="s">
         <v>92</v>
       </c>
       <c r="Q8" t="s">
+        <v>140</v>
+      </c>
+      <c r="R8">
+        <v>10</v>
+      </c>
+      <c r="S8" t="s">
         <v>141</v>
       </c>
-      <c r="R8" t="s">
+      <c r="T8" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>142</v>
       </c>
-      <c r="S8" t="s">
+      <c r="B9" t="s">
         <v>143</v>
       </c>
-      <c r="T8" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="9" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="C9" t="s">
+        <v>143</v>
+      </c>
+      <c r="D9" t="s">
         <v>144</v>
-      </c>
-      <c r="B9" t="s">
-        <v>145</v>
-      </c>
-      <c r="C9" t="s">
-        <v>145</v>
-      </c>
-      <c r="D9" t="s">
-        <v>146</v>
       </c>
       <c r="E9" t="s">
         <v>86</v>
@@ -2160,7 +2154,7 @@
         <v>0.5</v>
       </c>
       <c r="I9" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="J9">
         <v>36722.0625</v>
@@ -2172,42 +2166,42 @@
         <v>6.1</v>
       </c>
       <c r="M9" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="N9" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="O9" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="P9" t="s">
         <v>92</v>
       </c>
       <c r="Q9" t="s">
+        <v>146</v>
+      </c>
+      <c r="R9">
+        <v>10</v>
+      </c>
+      <c r="S9" t="s">
+        <v>147</v>
+      </c>
+      <c r="T9" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>148</v>
       </c>
-      <c r="R9" t="s">
-        <v>142</v>
-      </c>
-      <c r="S9" t="s">
+      <c r="B10" t="s">
+        <v>143</v>
+      </c>
+      <c r="C10" t="s">
+        <v>143</v>
+      </c>
+      <c r="D10" t="s">
         <v>149</v>
-      </c>
-      <c r="T9" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>150</v>
-      </c>
-      <c r="B10" t="s">
-        <v>145</v>
-      </c>
-      <c r="C10" t="s">
-        <v>145</v>
-      </c>
-      <c r="D10" t="s">
-        <v>151</v>
       </c>
       <c r="E10" t="s">
         <v>86</v>
@@ -2222,7 +2216,7 @@
         <v>0.5</v>
       </c>
       <c r="I10" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="J10">
         <v>36708.292361111111</v>
@@ -2234,42 +2228,42 @@
         <v>6.1</v>
       </c>
       <c r="M10" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="N10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="O10" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="P10" t="s">
         <v>92</v>
       </c>
       <c r="Q10" t="s">
-        <v>148</v>
-      </c>
-      <c r="R10" t="s">
-        <v>142</v>
+        <v>146</v>
+      </c>
+      <c r="R10">
+        <v>10</v>
       </c>
       <c r="S10" t="s">
+        <v>150</v>
+      </c>
+      <c r="T10" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>151</v>
+      </c>
+      <c r="B11" t="s">
         <v>152</v>
       </c>
-      <c r="T10" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="C11" t="s">
+        <v>152</v>
+      </c>
+      <c r="D11" t="s">
         <v>153</v>
-      </c>
-      <c r="B11" t="s">
-        <v>154</v>
-      </c>
-      <c r="C11" t="s">
-        <v>154</v>
-      </c>
-      <c r="D11" t="s">
-        <v>155</v>
       </c>
       <c r="E11" t="s">
         <v>86</v>
@@ -2284,7 +2278,7 @@
         <v>0.5</v>
       </c>
       <c r="I11" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="J11">
         <v>36830</v>
@@ -2296,39 +2290,39 @@
         <v>4.8</v>
       </c>
       <c r="M11" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="N11" t="s">
         <v>90</v>
       </c>
       <c r="O11" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="P11" t="s">
         <v>92</v>
       </c>
       <c r="Q11" t="s">
+        <v>157</v>
+      </c>
+      <c r="R11">
+        <v>0</v>
+      </c>
+      <c r="S11" t="s">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>159</v>
       </c>
-      <c r="R11" t="s">
-        <v>102</v>
-      </c>
-      <c r="S11" t="s">
+      <c r="B12" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="12" spans="1:21" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="C12" t="s">
+        <v>160</v>
+      </c>
+      <c r="D12" t="s">
         <v>161</v>
-      </c>
-      <c r="B12" t="s">
-        <v>162</v>
-      </c>
-      <c r="C12" t="s">
-        <v>162</v>
-      </c>
-      <c r="D12" t="s">
-        <v>163</v>
       </c>
       <c r="E12" t="s">
         <v>86</v>
@@ -2355,28 +2349,28 @@
         <v>6.5</v>
       </c>
       <c r="M12" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="N12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="O12" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="P12" t="s">
         <v>92</v>
       </c>
       <c r="Q12" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="R12">
         <v>1.9</v>
       </c>
       <c r="S12" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="T12" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="U12">
         <v>123487</v>
@@ -2385,7 +2379,7 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:U7 A11:U12 A8:H8 J8:U8 A9:H9 J9:U9 A10:H10 J10:U10" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:U2 A12:U12 A8:H8 J8:Q8 A9:H9 J9:Q9 A10:H10 J10:Q10 A5:U7 A3:Q3 S3:U3 A4:Q4 S4:U4 S8:U8 S9:U9 S10:U10 A11:Q11 S11:U11" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -2393,55 +2387,55 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:N12"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>65</v>
       </c>
       <c r="B1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C1" t="s">
+        <v>168</v>
+      </c>
+      <c r="D1" t="s">
         <v>169</v>
-      </c>
-      <c r="C1" t="s">
-        <v>170</v>
-      </c>
-      <c r="D1" t="s">
-        <v>171</v>
       </c>
       <c r="E1" t="s">
         <v>30</v>
       </c>
       <c r="F1" t="s">
+        <v>170</v>
+      </c>
+      <c r="G1" t="s">
+        <v>171</v>
+      </c>
+      <c r="H1" t="s">
         <v>172</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>173</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>174</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>175</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>176</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>177</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>178</v>
       </c>
-      <c r="M1" t="s">
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>179</v>
-      </c>
-      <c r="N1" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="2" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>181</v>
       </c>
       <c r="B2" t="s">
         <v>86</v>
@@ -2453,7 +2447,7 @@
         <v>0.25</v>
       </c>
       <c r="E2" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="F2">
         <v>2017</v>
@@ -2465,16 +2459,16 @@
         <v>80936</v>
       </c>
       <c r="I2" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="J2" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="K2">
         <v>569</v>
       </c>
       <c r="L2" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="M2">
         <v>11.087</v>
@@ -2483,9 +2477,9 @@
         <v>53.881999999999998</v>
       </c>
     </row>
-    <row r="3" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B3" t="s">
         <v>86</v>
@@ -2509,16 +2503,16 @@
         <v>80936</v>
       </c>
       <c r="I3" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="J3" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="K3">
         <v>569</v>
       </c>
       <c r="L3" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="M3">
         <v>104.991</v>
@@ -2527,9 +2521,9 @@
         <v>12.565</v>
       </c>
     </row>
-    <row r="4" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B4" t="s">
         <v>86</v>
@@ -2553,16 +2547,16 @@
         <v>80936</v>
       </c>
       <c r="I4" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="J4" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="K4">
         <v>569</v>
       </c>
       <c r="L4" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="M4">
         <v>11.087</v>
@@ -2571,9 +2565,9 @@
         <v>53.881999999999998</v>
       </c>
     </row>
-    <row r="5" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B5" t="s">
         <v>86</v>
@@ -2585,7 +2579,7 @@
         <v>0.25</v>
       </c>
       <c r="E5" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="F5">
         <v>2017</v>
@@ -2597,16 +2591,16 @@
         <v>80936</v>
       </c>
       <c r="I5" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="J5" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="K5">
         <v>569</v>
       </c>
       <c r="L5" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="M5">
         <v>11.087</v>
@@ -2615,9 +2609,9 @@
         <v>53.881999999999998</v>
       </c>
     </row>
-    <row r="6" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B6" t="s">
         <v>86</v>
@@ -2641,16 +2635,16 @@
         <v>80936</v>
       </c>
       <c r="I6" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="J6" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="K6">
         <v>569</v>
       </c>
       <c r="L6" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="M6">
         <v>11.087</v>
@@ -2659,9 +2653,9 @@
         <v>53.881999999999998</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B7" t="s">
         <v>86</v>
@@ -2673,7 +2667,7 @@
         <v>0.25</v>
       </c>
       <c r="E7" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="F7">
         <v>2017</v>
@@ -2685,16 +2679,16 @@
         <v>80936</v>
       </c>
       <c r="I7" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="J7" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="K7">
         <v>569</v>
       </c>
       <c r="L7" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="M7">
         <v>11.087</v>
@@ -2703,9 +2697,9 @@
         <v>53.881999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B8" t="s">
         <v>86</v>
@@ -2717,7 +2711,7 @@
         <v>0.75</v>
       </c>
       <c r="E8" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="F8">
         <v>2017</v>
@@ -2729,16 +2723,16 @@
         <v>18686</v>
       </c>
       <c r="I8" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="J8" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="K8">
         <v>289</v>
       </c>
       <c r="L8" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="M8">
         <v>65.5</v>
@@ -2747,9 +2741,9 @@
         <v>40.996000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B9" t="s">
         <v>86</v>
@@ -2773,16 +2767,16 @@
         <v>87604</v>
       </c>
       <c r="I9" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="J9" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="K9">
         <v>259</v>
       </c>
       <c r="L9" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="M9">
         <v>-50.104999999999997</v>
@@ -2791,12 +2785,12 @@
         <v>-21.917000000000002</v>
       </c>
     </row>
-    <row r="10" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C10">
         <v>2</v>
@@ -2817,16 +2811,16 @@
         <v>142608</v>
       </c>
       <c r="I10" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="J10" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="K10">
         <v>277</v>
       </c>
       <c r="L10" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="M10">
         <v>144.5</v>
@@ -2835,12 +2829,12 @@
         <v>-33.5</v>
       </c>
     </row>
-    <row r="11" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B11" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C11">
         <v>2</v>
@@ -2849,7 +2843,7 @@
         <v>1.5</v>
       </c>
       <c r="E11" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="F11">
         <v>2018</v>
@@ -2861,16 +2855,16 @@
         <v>68692</v>
       </c>
       <c r="I11" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="J11" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="K11">
         <v>177</v>
       </c>
       <c r="L11" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="M11">
         <v>46.463999999999999</v>
@@ -2879,9 +2873,9 @@
         <v>-19.498000000000001</v>
       </c>
     </row>
-    <row r="12" spans="1:14" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B12" t="s">
         <v>86</v>
@@ -2905,16 +2899,16 @@
         <v>104035</v>
       </c>
       <c r="I12" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="J12" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="K12">
         <v>224</v>
       </c>
       <c r="L12" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="M12">
         <v>-38.049999999999997</v>

</xml_diff>